<commit_message>
Update routing workbook for split jellyfish bypass topology
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1424,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23.48" customWidth="1" style="116" min="1" max="1"/>
@@ -2154,6 +2154,27 @@
       </c>
       <c r="B49" s="161" t="n">
         <v>0.039</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="116" t="inlineStr">
+        <is>
+          <t>Q_jelly_cap_m3s</t>
+        </is>
+      </c>
+      <c r="B50" s="116">
+        <f>B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="116" t="inlineStr">
+        <is>
+          <t>Rendement_retour_jelly</t>
+        </is>
+      </c>
+      <c r="B51" s="116" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2775,6 +2796,10 @@
     <col width="13.1" customWidth="1" style="116" min="10" max="10"/>
     <col width="8.220000000000001" customWidth="1" style="116" min="14" max="14"/>
     <col width="9.48" customWidth="1" style="116" min="15" max="15"/>
+    <col width="9.48" customWidth="1" style="117" min="16" max="16"/>
+    <col width="9.48" customWidth="1" style="117" min="17" max="17"/>
+    <col width="9.48" customWidth="1" style="117" min="18" max="18"/>
+    <col width="9.48" customWidth="1" style="117" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.6" customHeight="1" s="117">
@@ -2805,7 +2830,7 @@
       </c>
       <c r="F1" s="167" t="inlineStr">
         <is>
-          <t>Debit_Q12_vers_puisard_m3s</t>
+          <t>Q_RP_total_m3s</t>
         </is>
       </c>
       <c r="G1" s="169" t="inlineStr">
@@ -2853,7 +2878,26 @@
           <t>Cumul_demarrages</t>
         </is>
       </c>
-      <c r="P1" s="167" t="n"/>
+      <c r="P1" s="170" t="inlineStr">
+        <is>
+          <t>Q_jelly_in_m3s</t>
+        </is>
+      </c>
+      <c r="Q1" s="170" t="inlineStr">
+        <is>
+          <t>Q_bypass_m3s</t>
+        </is>
+      </c>
+      <c r="R1" s="170" t="inlineStr">
+        <is>
+          <t>Q_jelly_out_m3s</t>
+        </is>
+      </c>
+      <c r="S1" s="170" t="inlineStr">
+        <is>
+          <t>Q_in_poste_m3s</t>
+        </is>
+      </c>
       <c r="V1" s="116" t="inlineStr">
         <is>
           <t>BlockDepth_mm</t>
@@ -2910,6 +2954,18 @@
       <c r="O2" s="116" t="n">
         <v>0</v>
       </c>
+      <c r="P2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" s="116" t="n">
         <v>1</v>
       </c>
@@ -2948,11 +3004,11 @@
         <v/>
       </c>
       <c r="H3" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H2+(F3-L3-I3)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H2+(S3-M3-I3)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I3" s="178">
-        <f>MAX(0,(H2+(F3-L3)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H2+(S3-M3)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J3" s="178">
@@ -2968,7 +3024,7 @@
         <v/>
       </c>
       <c r="M3" s="177">
-        <f>MIN( L3, H2/Inputs!$B$9 + F3 )</f>
+        <f>MIN(L3,H2/Inputs!$B$9+S3)</f>
         <v/>
       </c>
       <c r="N3" s="170">
@@ -2977,6 +3033,22 @@
       </c>
       <c r="O3" s="170">
         <f>O2 + N3</f>
+        <v/>
+      </c>
+      <c r="P3" s="116">
+        <f>MIN(F3,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q3" s="116">
+        <f>MAX(0,F3-P3)</f>
+        <v/>
+      </c>
+      <c r="R3" s="116">
+        <f>P3*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S3" s="116">
+        <f>Q3+R3</f>
         <v/>
       </c>
       <c r="U3" s="116" t="n">
@@ -3017,11 +3089,11 @@
         <v/>
       </c>
       <c r="H4" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H3+(F4-L4-I4)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H3+(S4-M4-I4)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I4" s="178">
-        <f>MAX(0,(H3+(F4-L4)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H3+(S4-M4)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J4" s="178">
@@ -3037,7 +3109,7 @@
         <v/>
       </c>
       <c r="M4" s="177">
-        <f>MIN( L4, H3/Inputs!$B$9 + F4 )</f>
+        <f>MIN(L4,H3/Inputs!$B$9+S4)</f>
         <v/>
       </c>
       <c r="N4" s="170">
@@ -3046,6 +3118,22 @@
       </c>
       <c r="O4" s="170">
         <f>O3 + N4</f>
+        <v/>
+      </c>
+      <c r="P4" s="116">
+        <f>MIN(F4,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="116">
+        <f>MAX(0,F4-P4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="116">
+        <f>P4*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S4" s="116">
+        <f>Q4+R4</f>
         <v/>
       </c>
       <c r="U4" s="116" t="n">
@@ -3086,11 +3174,11 @@
         <v/>
       </c>
       <c r="H5" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H4+(F5-L5-I5)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H4+(S5-M5-I5)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I5" s="178">
-        <f>MAX(0,(H4+(F5-L5)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H4+(S5-M5)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J5" s="178">
@@ -3106,7 +3194,7 @@
         <v/>
       </c>
       <c r="M5" s="177">
-        <f>MIN( L5, H4/Inputs!$B$9 + F5 )</f>
+        <f>MIN(L5,H4/Inputs!$B$9+S5)</f>
         <v/>
       </c>
       <c r="N5" s="170">
@@ -3115,6 +3203,22 @@
       </c>
       <c r="O5" s="170">
         <f>O4 + N5</f>
+        <v/>
+      </c>
+      <c r="P5" s="116">
+        <f>MIN(F5,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="116">
+        <f>MAX(0,F5-P5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="116">
+        <f>P5*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S5" s="116">
+        <f>Q5+R5</f>
         <v/>
       </c>
       <c r="U5" s="116" t="n">
@@ -3155,11 +3259,11 @@
         <v/>
       </c>
       <c r="H6" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H5+(F6-L6-I6)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H5+(S6-M6-I6)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I6" s="178">
-        <f>MAX(0,(H5+(F6-L6)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H5+(S6-M6)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J6" s="178">
@@ -3175,7 +3279,7 @@
         <v/>
       </c>
       <c r="M6" s="177">
-        <f>MIN( L6, H5/Inputs!$B$9 + F6 )</f>
+        <f>MIN(L6,H5/Inputs!$B$9+S6)</f>
         <v/>
       </c>
       <c r="N6" s="170">
@@ -3184,6 +3288,22 @@
       </c>
       <c r="O6" s="170">
         <f>O5 + N6</f>
+        <v/>
+      </c>
+      <c r="P6" s="116">
+        <f>MIN(F6,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="116">
+        <f>MAX(0,F6-P6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="116">
+        <f>P6*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S6" s="116">
+        <f>Q6+R6</f>
         <v/>
       </c>
       <c r="U6" s="116" t="n">
@@ -3224,11 +3344,11 @@
         <v/>
       </c>
       <c r="H7" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H6+(F7-L7-I7)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H6+(S7-M7-I7)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I7" s="178">
-        <f>MAX(0,(H6+(F7-L7)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H6+(S7-M7)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J7" s="178">
@@ -3244,7 +3364,7 @@
         <v/>
       </c>
       <c r="M7" s="177">
-        <f>MIN( L7, H6/Inputs!$B$9 + F7 )</f>
+        <f>MIN(L7,H6/Inputs!$B$9+S7)</f>
         <v/>
       </c>
       <c r="N7" s="170">
@@ -3253,6 +3373,22 @@
       </c>
       <c r="O7" s="170">
         <f>O6 + N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="116">
+        <f>MIN(F7,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="116">
+        <f>MAX(0,F7-P7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="116">
+        <f>P7*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S7" s="116">
+        <f>Q7+R7</f>
         <v/>
       </c>
       <c r="U7" s="116" t="n">
@@ -3293,11 +3429,11 @@
         <v/>
       </c>
       <c r="H8" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H7+(F8-L8-I8)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H7+(S8-M8-I8)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I8" s="178">
-        <f>MAX(0,(H7+(F8-L8)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H7+(S8-M8)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J8" s="178">
@@ -3313,7 +3449,7 @@
         <v/>
       </c>
       <c r="M8" s="177">
-        <f>MIN( L8, H7/Inputs!$B$9 + F8 )</f>
+        <f>MIN(L8,H7/Inputs!$B$9+S8)</f>
         <v/>
       </c>
       <c r="N8" s="170">
@@ -3322,6 +3458,22 @@
       </c>
       <c r="O8" s="170">
         <f>O7 + N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="116">
+        <f>MIN(F8,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="116">
+        <f>MAX(0,F8-P8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="116">
+        <f>P8*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S8" s="116">
+        <f>Q8+R8</f>
         <v/>
       </c>
       <c r="U8" s="116" t="n">
@@ -3362,11 +3514,11 @@
         <v/>
       </c>
       <c r="H9" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H8+(F9-L9-I9)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H8+(S9-M9-I9)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I9" s="178">
-        <f>MAX(0,(H8+(F9-L9)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H8+(S9-M9)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J9" s="178">
@@ -3382,7 +3534,7 @@
         <v/>
       </c>
       <c r="M9" s="177">
-        <f>MIN( L9, H8/Inputs!$B$9 + F9 )</f>
+        <f>MIN(L9,H8/Inputs!$B$9+S9)</f>
         <v/>
       </c>
       <c r="N9" s="170">
@@ -3391,6 +3543,22 @@
       </c>
       <c r="O9" s="170">
         <f>O8 + N9</f>
+        <v/>
+      </c>
+      <c r="P9" s="116">
+        <f>MIN(F9,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="116">
+        <f>MAX(0,F9-P9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="116">
+        <f>P9*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S9" s="116">
+        <f>Q9+R9</f>
         <v/>
       </c>
       <c r="U9" s="116" t="n">
@@ -3431,11 +3599,11 @@
         <v/>
       </c>
       <c r="H10" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H9+(F10-L10-I10)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H9+(S10-M10-I10)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I10" s="178">
-        <f>MAX(0,(H9+(F10-L10)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H9+(S10-M10)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J10" s="178">
@@ -3451,7 +3619,7 @@
         <v/>
       </c>
       <c r="M10" s="177">
-        <f>MIN( L10, H9/Inputs!$B$9 + F10 )</f>
+        <f>MIN(L10,H9/Inputs!$B$9+S10)</f>
         <v/>
       </c>
       <c r="N10" s="170">
@@ -3460,6 +3628,22 @@
       </c>
       <c r="O10" s="170">
         <f>O9 + N10</f>
+        <v/>
+      </c>
+      <c r="P10" s="116">
+        <f>MIN(F10,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="116">
+        <f>MAX(0,F10-P10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="116">
+        <f>P10*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S10" s="116">
+        <f>Q10+R10</f>
         <v/>
       </c>
       <c r="U10" s="116" t="n">
@@ -3500,11 +3684,11 @@
         <v/>
       </c>
       <c r="H11" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H10+(F11-L11-I11)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H10+(S11-M11-I11)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I11" s="178">
-        <f>MAX(0,(H10+(F11-L11)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H10+(S11-M11)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J11" s="178">
@@ -3520,7 +3704,7 @@
         <v/>
       </c>
       <c r="M11" s="177">
-        <f>MIN( L11, H10/Inputs!$B$9 + F11 )</f>
+        <f>MIN(L11,H10/Inputs!$B$9+S11)</f>
         <v/>
       </c>
       <c r="N11" s="170">
@@ -3529,6 +3713,22 @@
       </c>
       <c r="O11" s="170">
         <f>O10 + N11</f>
+        <v/>
+      </c>
+      <c r="P11" s="116">
+        <f>MIN(F11,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="116">
+        <f>MAX(0,F11-P11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="116">
+        <f>P11*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S11" s="116">
+        <f>Q11+R11</f>
         <v/>
       </c>
       <c r="U11" s="116" t="n">
@@ -3569,11 +3769,11 @@
         <v/>
       </c>
       <c r="H12" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H11+(F12-L12-I12)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H11+(S12-M12-I12)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I12" s="178">
-        <f>MAX(0,(H11+(F12-L12)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H11+(S12-M12)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J12" s="178">
@@ -3589,7 +3789,7 @@
         <v/>
       </c>
       <c r="M12" s="177">
-        <f>MIN( L12, H11/Inputs!$B$9 + F12 )</f>
+        <f>MIN(L12,H11/Inputs!$B$9+S12)</f>
         <v/>
       </c>
       <c r="N12" s="170">
@@ -3598,6 +3798,22 @@
       </c>
       <c r="O12" s="170">
         <f>O11 + N12</f>
+        <v/>
+      </c>
+      <c r="P12" s="116">
+        <f>MIN(F12,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="116">
+        <f>MAX(0,F12-P12)</f>
+        <v/>
+      </c>
+      <c r="R12" s="116">
+        <f>P12*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S12" s="116">
+        <f>Q12+R12</f>
         <v/>
       </c>
       <c r="U12" s="116" t="n">
@@ -3638,11 +3854,11 @@
         <v/>
       </c>
       <c r="H13" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H12+(F13-L13-I13)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H12+(S13-M13-I13)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I13" s="178">
-        <f>MAX(0,(H12+(F13-L13)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H12+(S13-M13)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J13" s="178">
@@ -3658,7 +3874,7 @@
         <v/>
       </c>
       <c r="M13" s="177">
-        <f>MIN( L13, H12/Inputs!$B$9 + F13 )</f>
+        <f>MIN(L13,H12/Inputs!$B$9+S13)</f>
         <v/>
       </c>
       <c r="N13" s="170">
@@ -3667,6 +3883,22 @@
       </c>
       <c r="O13" s="170">
         <f>O12 + N13</f>
+        <v/>
+      </c>
+      <c r="P13" s="116">
+        <f>MIN(F13,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="116">
+        <f>MAX(0,F13-P13)</f>
+        <v/>
+      </c>
+      <c r="R13" s="116">
+        <f>P13*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S13" s="116">
+        <f>Q13+R13</f>
         <v/>
       </c>
       <c r="U13" s="116" t="n">
@@ -3707,11 +3939,11 @@
         <v/>
       </c>
       <c r="H14" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H13+(F14-L14-I14)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H13+(S14-M14-I14)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I14" s="178">
-        <f>MAX(0,(H13+(F14-L14)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H13+(S14-M14)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J14" s="178">
@@ -3727,7 +3959,7 @@
         <v/>
       </c>
       <c r="M14" s="177">
-        <f>MIN( L14, H13/Inputs!$B$9 + F14 )</f>
+        <f>MIN(L14,H13/Inputs!$B$9+S14)</f>
         <v/>
       </c>
       <c r="N14" s="170">
@@ -3736,6 +3968,22 @@
       </c>
       <c r="O14" s="170">
         <f>O13 + N14</f>
+        <v/>
+      </c>
+      <c r="P14" s="116">
+        <f>MIN(F14,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="116">
+        <f>MAX(0,F14-P14)</f>
+        <v/>
+      </c>
+      <c r="R14" s="116">
+        <f>P14*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S14" s="116">
+        <f>Q14+R14</f>
         <v/>
       </c>
     </row>
@@ -5342,7 +5590,7 @@
           <t>NOTE</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="116" t="inlineStr">
         <is>
           <t>Valider K Jellyfish et K regulateur sur fiches fabricants.</t>
         </is>

</xml_diff>

<commit_message>
sync: take updated routing workbook from cursor branch
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1424,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23.48" customWidth="1" style="116" min="1" max="1"/>
@@ -2154,6 +2154,27 @@
       </c>
       <c r="B49" s="161" t="n">
         <v>0.039</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="116" t="inlineStr">
+        <is>
+          <t>Q_jelly_cap_m3s</t>
+        </is>
+      </c>
+      <c r="B50" s="116">
+        <f>B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="116" t="inlineStr">
+        <is>
+          <t>Rendement_retour_jelly</t>
+        </is>
+      </c>
+      <c r="B51" s="116" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2775,6 +2796,10 @@
     <col width="13.1" customWidth="1" style="116" min="10" max="10"/>
     <col width="8.220000000000001" customWidth="1" style="116" min="14" max="14"/>
     <col width="9.48" customWidth="1" style="116" min="15" max="15"/>
+    <col width="9.48" customWidth="1" style="117" min="16" max="16"/>
+    <col width="9.48" customWidth="1" style="117" min="17" max="17"/>
+    <col width="9.48" customWidth="1" style="117" min="18" max="18"/>
+    <col width="9.48" customWidth="1" style="117" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.6" customHeight="1" s="117">
@@ -2805,7 +2830,7 @@
       </c>
       <c r="F1" s="167" t="inlineStr">
         <is>
-          <t>Debit_Q12_vers_puisard_m3s</t>
+          <t>Q_RP_total_m3s</t>
         </is>
       </c>
       <c r="G1" s="169" t="inlineStr">
@@ -2853,7 +2878,26 @@
           <t>Cumul_demarrages</t>
         </is>
       </c>
-      <c r="P1" s="167" t="n"/>
+      <c r="P1" s="170" t="inlineStr">
+        <is>
+          <t>Q_jelly_in_m3s</t>
+        </is>
+      </c>
+      <c r="Q1" s="170" t="inlineStr">
+        <is>
+          <t>Q_bypass_m3s</t>
+        </is>
+      </c>
+      <c r="R1" s="170" t="inlineStr">
+        <is>
+          <t>Q_jelly_out_m3s</t>
+        </is>
+      </c>
+      <c r="S1" s="170" t="inlineStr">
+        <is>
+          <t>Q_in_poste_m3s</t>
+        </is>
+      </c>
       <c r="V1" s="116" t="inlineStr">
         <is>
           <t>BlockDepth_mm</t>
@@ -2910,6 +2954,18 @@
       <c r="O2" s="116" t="n">
         <v>0</v>
       </c>
+      <c r="P2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="116" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="U2" s="116" t="n">
         <v>1</v>
       </c>
@@ -2948,11 +3004,11 @@
         <v/>
       </c>
       <c r="H3" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H2+(F3-L3-I3)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H2+(S3-M3-I3)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I3" s="178">
-        <f>MAX(0,(H2+(F3-L3)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H2+(S3-M3)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J3" s="178">
@@ -2968,7 +3024,7 @@
         <v/>
       </c>
       <c r="M3" s="177">
-        <f>MIN( L3, H2/Inputs!$B$9 + F3 )</f>
+        <f>MIN(L3,H2/Inputs!$B$9+S3)</f>
         <v/>
       </c>
       <c r="N3" s="170">
@@ -2977,6 +3033,22 @@
       </c>
       <c r="O3" s="170">
         <f>O2 + N3</f>
+        <v/>
+      </c>
+      <c r="P3" s="116">
+        <f>MIN(F3,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q3" s="116">
+        <f>MAX(0,F3-P3)</f>
+        <v/>
+      </c>
+      <c r="R3" s="116">
+        <f>P3*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S3" s="116">
+        <f>Q3+R3</f>
         <v/>
       </c>
       <c r="U3" s="116" t="n">
@@ -3017,11 +3089,11 @@
         <v/>
       </c>
       <c r="H4" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H3+(F4-L4-I4)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H3+(S4-M4-I4)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I4" s="178">
-        <f>MAX(0,(H3+(F4-L4)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H3+(S4-M4)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J4" s="178">
@@ -3037,7 +3109,7 @@
         <v/>
       </c>
       <c r="M4" s="177">
-        <f>MIN( L4, H3/Inputs!$B$9 + F4 )</f>
+        <f>MIN(L4,H3/Inputs!$B$9+S4)</f>
         <v/>
       </c>
       <c r="N4" s="170">
@@ -3046,6 +3118,22 @@
       </c>
       <c r="O4" s="170">
         <f>O3 + N4</f>
+        <v/>
+      </c>
+      <c r="P4" s="116">
+        <f>MIN(F4,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="116">
+        <f>MAX(0,F4-P4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="116">
+        <f>P4*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S4" s="116">
+        <f>Q4+R4</f>
         <v/>
       </c>
       <c r="U4" s="116" t="n">
@@ -3086,11 +3174,11 @@
         <v/>
       </c>
       <c r="H5" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H4+(F5-L5-I5)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H4+(S5-M5-I5)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I5" s="178">
-        <f>MAX(0,(H4+(F5-L5)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H4+(S5-M5)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J5" s="178">
@@ -3106,7 +3194,7 @@
         <v/>
       </c>
       <c r="M5" s="177">
-        <f>MIN( L5, H4/Inputs!$B$9 + F5 )</f>
+        <f>MIN(L5,H4/Inputs!$B$9+S5)</f>
         <v/>
       </c>
       <c r="N5" s="170">
@@ -3115,6 +3203,22 @@
       </c>
       <c r="O5" s="170">
         <f>O4 + N5</f>
+        <v/>
+      </c>
+      <c r="P5" s="116">
+        <f>MIN(F5,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="116">
+        <f>MAX(0,F5-P5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="116">
+        <f>P5*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S5" s="116">
+        <f>Q5+R5</f>
         <v/>
       </c>
       <c r="U5" s="116" t="n">
@@ -3155,11 +3259,11 @@
         <v/>
       </c>
       <c r="H6" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H5+(F6-L6-I6)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H5+(S6-M6-I6)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I6" s="178">
-        <f>MAX(0,(H5+(F6-L6)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H5+(S6-M6)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J6" s="178">
@@ -3175,7 +3279,7 @@
         <v/>
       </c>
       <c r="M6" s="177">
-        <f>MIN( L6, H5/Inputs!$B$9 + F6 )</f>
+        <f>MIN(L6,H5/Inputs!$B$9+S6)</f>
         <v/>
       </c>
       <c r="N6" s="170">
@@ -3184,6 +3288,22 @@
       </c>
       <c r="O6" s="170">
         <f>O5 + N6</f>
+        <v/>
+      </c>
+      <c r="P6" s="116">
+        <f>MIN(F6,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="116">
+        <f>MAX(0,F6-P6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="116">
+        <f>P6*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S6" s="116">
+        <f>Q6+R6</f>
         <v/>
       </c>
       <c r="U6" s="116" t="n">
@@ -3224,11 +3344,11 @@
         <v/>
       </c>
       <c r="H7" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H6+(F7-L7-I7)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H6+(S7-M7-I7)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I7" s="178">
-        <f>MAX(0,(H6+(F7-L7)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H6+(S7-M7)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J7" s="178">
@@ -3244,7 +3364,7 @@
         <v/>
       </c>
       <c r="M7" s="177">
-        <f>MIN( L7, H6/Inputs!$B$9 + F7 )</f>
+        <f>MIN(L7,H6/Inputs!$B$9+S7)</f>
         <v/>
       </c>
       <c r="N7" s="170">
@@ -3253,6 +3373,22 @@
       </c>
       <c r="O7" s="170">
         <f>O6 + N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="116">
+        <f>MIN(F7,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="116">
+        <f>MAX(0,F7-P7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="116">
+        <f>P7*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S7" s="116">
+        <f>Q7+R7</f>
         <v/>
       </c>
       <c r="U7" s="116" t="n">
@@ -3293,11 +3429,11 @@
         <v/>
       </c>
       <c r="H8" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H7+(F8-L8-I8)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H7+(S8-M8-I8)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I8" s="178">
-        <f>MAX(0,(H7+(F8-L8)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H7+(S8-M8)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J8" s="178">
@@ -3313,7 +3449,7 @@
         <v/>
       </c>
       <c r="M8" s="177">
-        <f>MIN( L8, H7/Inputs!$B$9 + F8 )</f>
+        <f>MIN(L8,H7/Inputs!$B$9+S8)</f>
         <v/>
       </c>
       <c r="N8" s="170">
@@ -3322,6 +3458,22 @@
       </c>
       <c r="O8" s="170">
         <f>O7 + N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="116">
+        <f>MIN(F8,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="116">
+        <f>MAX(0,F8-P8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="116">
+        <f>P8*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S8" s="116">
+        <f>Q8+R8</f>
         <v/>
       </c>
       <c r="U8" s="116" t="n">
@@ -3362,11 +3514,11 @@
         <v/>
       </c>
       <c r="H9" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H8+(F9-L9-I9)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H8+(S9-M9-I9)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I9" s="178">
-        <f>MAX(0,(H8+(F9-L9)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H8+(S9-M9)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J9" s="178">
@@ -3382,7 +3534,7 @@
         <v/>
       </c>
       <c r="M9" s="177">
-        <f>MIN( L9, H8/Inputs!$B$9 + F9 )</f>
+        <f>MIN(L9,H8/Inputs!$B$9+S9)</f>
         <v/>
       </c>
       <c r="N9" s="170">
@@ -3391,6 +3543,22 @@
       </c>
       <c r="O9" s="170">
         <f>O8 + N9</f>
+        <v/>
+      </c>
+      <c r="P9" s="116">
+        <f>MIN(F9,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="116">
+        <f>MAX(0,F9-P9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="116">
+        <f>P9*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S9" s="116">
+        <f>Q9+R9</f>
         <v/>
       </c>
       <c r="U9" s="116" t="n">
@@ -3431,11 +3599,11 @@
         <v/>
       </c>
       <c r="H10" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H9+(F10-L10-I10)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H9+(S10-M10-I10)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I10" s="178">
-        <f>MAX(0,(H9+(F10-L10)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H9+(S10-M10)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J10" s="178">
@@ -3451,7 +3619,7 @@
         <v/>
       </c>
       <c r="M10" s="177">
-        <f>MIN( L10, H9/Inputs!$B$9 + F10 )</f>
+        <f>MIN(L10,H9/Inputs!$B$9+S10)</f>
         <v/>
       </c>
       <c r="N10" s="170">
@@ -3460,6 +3628,22 @@
       </c>
       <c r="O10" s="170">
         <f>O9 + N10</f>
+        <v/>
+      </c>
+      <c r="P10" s="116">
+        <f>MIN(F10,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="116">
+        <f>MAX(0,F10-P10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="116">
+        <f>P10*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S10" s="116">
+        <f>Q10+R10</f>
         <v/>
       </c>
       <c r="U10" s="116" t="n">
@@ -3500,11 +3684,11 @@
         <v/>
       </c>
       <c r="H11" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H10+(F11-L11-I11)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H10+(S11-M11-I11)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I11" s="178">
-        <f>MAX(0,(H10+(F11-L11)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H10+(S11-M11)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J11" s="178">
@@ -3520,7 +3704,7 @@
         <v/>
       </c>
       <c r="M11" s="177">
-        <f>MIN( L11, H10/Inputs!$B$9 + F11 )</f>
+        <f>MIN(L11,H10/Inputs!$B$9+S11)</f>
         <v/>
       </c>
       <c r="N11" s="170">
@@ -3529,6 +3713,22 @@
       </c>
       <c r="O11" s="170">
         <f>O10 + N11</f>
+        <v/>
+      </c>
+      <c r="P11" s="116">
+        <f>MIN(F11,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="116">
+        <f>MAX(0,F11-P11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="116">
+        <f>P11*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S11" s="116">
+        <f>Q11+R11</f>
         <v/>
       </c>
       <c r="U11" s="116" t="n">
@@ -3569,11 +3769,11 @@
         <v/>
       </c>
       <c r="H12" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H11+(F12-L12-I12)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H11+(S12-M12-I12)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I12" s="178">
-        <f>MAX(0,(H11+(F12-L12)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H11+(S12-M12)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J12" s="178">
@@ -3589,7 +3789,7 @@
         <v/>
       </c>
       <c r="M12" s="177">
-        <f>MIN( L12, H11/Inputs!$B$9 + F12 )</f>
+        <f>MIN(L12,H11/Inputs!$B$9+S12)</f>
         <v/>
       </c>
       <c r="N12" s="170">
@@ -3598,6 +3798,22 @@
       </c>
       <c r="O12" s="170">
         <f>O11 + N12</f>
+        <v/>
+      </c>
+      <c r="P12" s="116">
+        <f>MIN(F12,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="116">
+        <f>MAX(0,F12-P12)</f>
+        <v/>
+      </c>
+      <c r="R12" s="116">
+        <f>P12*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S12" s="116">
+        <f>Q12+R12</f>
         <v/>
       </c>
       <c r="U12" s="116" t="n">
@@ -3638,11 +3854,11 @@
         <v/>
       </c>
       <c r="H13" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H12+(F13-L13-I13)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H12+(S13-M13-I13)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I13" s="178">
-        <f>MAX(0,(H12+(F13-L13)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H12+(S13-M13)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J13" s="178">
@@ -3658,7 +3874,7 @@
         <v/>
       </c>
       <c r="M13" s="177">
-        <f>MIN( L13, H12/Inputs!$B$9 + F13 )</f>
+        <f>MIN(L13,H12/Inputs!$B$9+S13)</f>
         <v/>
       </c>
       <c r="N13" s="170">
@@ -3667,6 +3883,22 @@
       </c>
       <c r="O13" s="170">
         <f>O12 + N13</f>
+        <v/>
+      </c>
+      <c r="P13" s="116">
+        <f>MIN(F13,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="116">
+        <f>MAX(0,F13-P13)</f>
+        <v/>
+      </c>
+      <c r="R13" s="116">
+        <f>P13*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S13" s="116">
+        <f>Q13+R13</f>
         <v/>
       </c>
       <c r="U13" s="116" t="n">
@@ -3707,11 +3939,11 @@
         <v/>
       </c>
       <c r="H14" s="178">
-        <f>MAX(0,MIN(Inputs!$B$44,H13+(F14-L14-I14)*Inputs!$B$9))</f>
+        <f>MAX(0,MIN(Inputs!$B$44,H13+(S14-M14-I14)*Inputs!$B$9))</f>
         <v/>
       </c>
       <c r="I14" s="178">
-        <f>MAX(0,(H13+(F14-L14)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
+        <f>MAX(0,(H13+(S14-M14)*Inputs!$B$9-Inputs!$B$44)/Inputs!$B$9)</f>
         <v/>
       </c>
       <c r="J14" s="178">
@@ -3727,7 +3959,7 @@
         <v/>
       </c>
       <c r="M14" s="177">
-        <f>MIN( L14, H13/Inputs!$B$9 + F14 )</f>
+        <f>MIN(L14,H13/Inputs!$B$9+S14)</f>
         <v/>
       </c>
       <c r="N14" s="170">
@@ -3736,6 +3968,22 @@
       </c>
       <c r="O14" s="170">
         <f>O13 + N14</f>
+        <v/>
+      </c>
+      <c r="P14" s="116">
+        <f>MIN(F14,Inputs!$B$50)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="116">
+        <f>MAX(0,F14-P14)</f>
+        <v/>
+      </c>
+      <c r="R14" s="116">
+        <f>P14*Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="S14" s="116">
+        <f>Q14+R14</f>
         <v/>
       </c>
     </row>
@@ -5342,7 +5590,7 @@
           <t>NOTE</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="116" t="inlineStr">
         <is>
           <t>Valider K Jellyfish et K regulateur sur fiches fabricants.</t>
         </is>

</xml_diff>

<commit_message>
Update minor-loss detail sheet for split DP-01 topology
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -5088,14 +5088,14 @@
     <row r="3">
       <c r="A3" s="231" t="inlineStr">
         <is>
-          <t>Configuration consideree: Toiture -&gt; StormBrixx -&gt; regard regulateur -&gt; branche Jellyfish / branche poste pompage.</t>
+          <t>Configuration consideree: StormBrixx -&gt; regard RP-01 (regulateur) -&gt; split vers poste direct et vers DP-01, puis retour DP-01 au poste.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="232" t="inlineStr">
         <is>
-          <t>IMPORTANT: Les K du regulateur et Jellyfish sont provisoires. Remplacer par les pertes de charge constructeur pour le dimensionnement final.</t>
+          <t>IMPORTANT: Les K du regulateur et du separateur dynamique sont provisoires. Remplacer par les pertes constructeur pour le dimensionnement final.</t>
         </is>
       </c>
     </row>
@@ -5204,17 +5204,18 @@
       </c>
       <c r="B10" s="237" t="inlineStr">
         <is>
-          <t>Bassin retention vers RP-01</t>
+          <t>StormBrixx vers regard RP-01 regulateur</t>
         </is>
       </c>
       <c r="C10" s="237" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E10" s="237" t="n">
-        <v>0.029</v>
+      <c r="E10" s="237">
+        <f>MAX(Routing!$F$2:$F$2000)</f>
+        <v/>
       </c>
       <c r="F10" s="238">
         <f>IF(D10&gt;0,PI()*(D10^2)/4,0)</f>
@@ -5249,7 +5250,7 @@
       </c>
       <c r="N10" s="237" t="inlineStr">
         <is>
-          <t>Conduite entree</t>
+          <t>Troncon commun amont</t>
         </is>
       </c>
       <c r="P10" s="235" t="inlineStr">
@@ -5271,7 +5272,7 @@
       </c>
       <c r="B11" s="237" t="inlineStr">
         <is>
-          <t>RP-01 vers regard regulateur</t>
+          <t>RP-01 vers poste de pompage (branche directe)</t>
         </is>
       </c>
       <c r="C11" s="237" t="n">
@@ -5280,8 +5281,9 @@
       <c r="D11" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E11" s="237" t="n">
-        <v>0.029</v>
+      <c r="E11" s="237">
+        <f>MAX(Routing!$Q$2:$Q$2000)</f>
+        <v/>
       </c>
       <c r="F11" s="238">
         <f>IF(D11&gt;0,PI()*(D11^2)/4,0)</f>
@@ -5316,16 +5318,16 @@
       </c>
       <c r="N11" s="237" t="inlineStr">
         <is>
-          <t>Collecteur principal</t>
+          <t>Branche directe vers poste</t>
         </is>
       </c>
       <c r="P11" s="239" t="inlineStr">
         <is>
-          <t>Vers Jellyfish (S1+S2+S3)</t>
+          <t>Chemin direct vers poste (S1+S2)</t>
         </is>
       </c>
       <c r="Q11" s="238">
-        <f>M10+M11+M12</f>
+        <f>M10+M11</f>
         <v/>
       </c>
     </row>
@@ -5337,7 +5339,7 @@
       </c>
       <c r="B12" s="237" t="inlineStr">
         <is>
-          <t>Regard regulateur vers DP-01 (Jellyfish)</t>
+          <t>RP-01 vers DP-01 separateur dynamique</t>
         </is>
       </c>
       <c r="C12" s="237" t="n">
@@ -5346,8 +5348,9 @@
       <c r="D12" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E12" s="237" t="n">
-        <v>0.029</v>
+      <c r="E12" s="237">
+        <f>MAX(Routing!$P$2:$P$2000)</f>
+        <v/>
       </c>
       <c r="F12" s="238">
         <f>IF(D12&gt;0,PI()*(D12^2)/4,0)</f>
@@ -5382,16 +5385,16 @@
       </c>
       <c r="N12" s="237" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Branche derivee vers separateur</t>
         </is>
       </c>
       <c r="P12" s="239" t="inlineStr">
         <is>
-          <t>Vers poste pompage (S1+S2+S4)</t>
+          <t>Chemin via separateur (S1+S3+S4)</t>
         </is>
       </c>
       <c r="Q12" s="238">
-        <f>M10+M11+M13</f>
+        <f>M10+M12+M13</f>
         <v/>
       </c>
     </row>
@@ -5403,17 +5406,18 @@
       </c>
       <c r="B13" s="237" t="inlineStr">
         <is>
-          <t>Regard regulateur vers poste pompage</t>
+          <t>DP-01 vers poste de pompage (retour)</t>
         </is>
       </c>
       <c r="C13" s="237" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="D13" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E13" s="237" t="n">
-        <v>0.164</v>
+      <c r="E13" s="237">
+        <f>MAX(Routing!$R$2:$R$2000)</f>
+        <v/>
       </c>
       <c r="F13" s="238">
         <f>IF(D13&gt;0,PI()*(D13^2)/4,0)</f>
@@ -5448,12 +5452,12 @@
       </c>
       <c r="N13" s="237" t="inlineStr">
         <is>
-          <t>Branche surverse (Q=163.8 L/s)</t>
+          <t>Retour du separateur vers poste</t>
         </is>
       </c>
       <c r="P13" s="239" t="inlineStr">
         <is>
-          <t>Refoulement pompe (S5)</t>
+          <t>Troncon poste vers RP-02 (S5)</t>
         </is>
       </c>
       <c r="Q13" s="238">
@@ -5469,17 +5473,18 @@
       </c>
       <c r="B14" s="237" t="inlineStr">
         <is>
-          <t>Ligne de refoulement poste pompage</t>
+          <t>Poste de pompage vers RP-02 avec clapet</t>
         </is>
       </c>
       <c r="C14" s="237" t="n">
-        <v>31.5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="237" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E14" s="237" t="n">
-        <v>0.039</v>
+        <v>0.3</v>
+      </c>
+      <c r="E14" s="237">
+        <f>MAX(Routing!$M$2:$M$2000)</f>
+        <v/>
       </c>
       <c r="F14" s="238">
         <f>IF(D14&gt;0,PI()*(D14^2)/4,0)</f>
@@ -5514,12 +5519,12 @@
       </c>
       <c r="N14" s="237" t="inlineStr">
         <is>
-          <t>Refoulement pompe (Q unitaire)</t>
+          <t>Aval poste vers RP-02</t>
         </is>
       </c>
       <c r="P14" s="239" t="inlineStr">
         <is>
-          <t>Exutoire gravitaire aval (S6)</t>
+          <t>Troncon aval gravitaire (S6)</t>
         </is>
       </c>
       <c r="Q14" s="238">
@@ -5535,17 +5540,18 @@
       </c>
       <c r="B15" s="237" t="inlineStr">
         <is>
-          <t>RP avec clapet vers exutoire gravite</t>
+          <t>RP-02 vers exutoire gravitaire</t>
         </is>
       </c>
       <c r="C15" s="237" t="n">
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="D15" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E15" s="237" t="n">
-        <v>0.039</v>
+      <c r="E15" s="237">
+        <f>E14</f>
+        <v/>
       </c>
       <c r="F15" s="238">
         <f>IF(D15&gt;0,PI()*(D15^2)/4,0)</f>
@@ -5580,7 +5586,7 @@
       </c>
       <c r="N15" s="237" t="inlineStr">
         <is>
-          <t>Troncon aval gravitaire</t>
+          <t>Troncon final a gravite</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5598,7 @@
       </c>
       <c r="Q17" s="116" t="inlineStr">
         <is>
-          <t>Valider K Jellyfish et K regulateur sur fiches fabricants.</t>
+          <t>Valider K regulateur, K separateur et K clapet RP-02 sur fiches fabricants.</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5644,7 @@
       </c>
       <c r="B21" s="237" t="inlineStr">
         <is>
-          <t>Entree brusque</t>
+          <t>Entree depuis StormBrixx</t>
         </is>
       </c>
       <c r="C21" s="237" t="n">
@@ -5660,14 +5666,14 @@
       </c>
       <c r="B22" s="237" t="inlineStr">
         <is>
-          <t>Coude 90 rayon court</t>
+          <t>Regard RP-01 (passage)</t>
         </is>
       </c>
       <c r="C22" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="237" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="238">
         <f>C22*D22</f>
@@ -5677,19 +5683,19 @@
     <row r="23">
       <c r="A23" s="237" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B23" s="237" t="inlineStr">
         <is>
-          <t>Regard traversant</t>
+          <t>Regulateur RP-01 (provisoire)</t>
         </is>
       </c>
       <c r="C23" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="237" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="E23" s="238">
         <f>C23*D23</f>
@@ -5704,14 +5710,14 @@
       </c>
       <c r="B24" s="237" t="inlineStr">
         <is>
-          <t>Coude 45</t>
+          <t>Te passage droit (vers branche directe)</t>
         </is>
       </c>
       <c r="C24" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="237" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E24" s="238">
         <f>C24*D24</f>
@@ -5721,19 +5727,19 @@
     <row r="25">
       <c r="A25" s="237" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B25" s="237" t="inlineStr">
         <is>
-          <t>Te derivation</t>
+          <t>Coude de raccordement vers poste</t>
         </is>
       </c>
       <c r="C25" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="237" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="E25" s="238">
         <f>C25*D25</f>
@@ -5748,14 +5754,14 @@
       </c>
       <c r="B26" s="237" t="inlineStr">
         <is>
-          <t>Equipement Jellyfish (provisoire)</t>
+          <t>Te derivation vers DP-01</t>
         </is>
       </c>
       <c r="C26" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="237" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E26" s="238">
         <f>C26*D26</f>
@@ -5765,19 +5771,19 @@
     <row r="27">
       <c r="A27" s="237" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B27" s="237" t="inlineStr">
         <is>
-          <t>Te passage droit</t>
+          <t>Entree separateur dynamique</t>
         </is>
       </c>
       <c r="C27" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="237" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="238">
         <f>C27*D27</f>
@@ -5792,14 +5798,14 @@
       </c>
       <c r="B28" s="237" t="inlineStr">
         <is>
-          <t>Regulateur Q-brake (provisoire)</t>
+          <t>Sortie separateur dynamique (provisoire)</t>
         </is>
       </c>
       <c r="C28" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="237" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E28" s="238">
         <f>C28*D28</f>
@@ -5809,19 +5815,19 @@
     <row r="29">
       <c r="A29" s="237" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B29" s="237" t="inlineStr">
         <is>
-          <t>Clapet anti-retour</t>
+          <t>Raccord retour vers poste</t>
         </is>
       </c>
       <c r="C29" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="237" t="n">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="E29" s="238">
         <f>C29*D29</f>
@@ -5836,14 +5842,14 @@
       </c>
       <c r="B30" s="237" t="inlineStr">
         <is>
-          <t>Vanne d'isolement ouverte</t>
+          <t>Clapet anti-retour RP-02</t>
         </is>
       </c>
       <c r="C30" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="237" t="n">
-        <v>0.2</v>
+        <v>2.5</v>
       </c>
       <c r="E30" s="238">
         <f>C30*D30</f>
@@ -5858,11 +5864,11 @@
       </c>
       <c r="B31" s="237" t="inlineStr">
         <is>
-          <t>Coude 90 (x2)</t>
+          <t>Coude 90</t>
         </is>
       </c>
       <c r="C31" s="237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="237" t="n">
         <v>0.9</v>
@@ -5880,7 +5886,7 @@
       </c>
       <c r="B32" s="237" t="inlineStr">
         <is>
-          <t>Sortie libre</t>
+          <t>Sortie libre a l'exutoire</t>
         </is>
       </c>
       <c r="C32" s="237" t="n">

</xml_diff>

<commit_message>
Link Inputs K coefficient to minor-loss detail analysis
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1800,8 +1800,9 @@
           <t>Coeff_pertes_singulieres_K_total</t>
         </is>
       </c>
-      <c r="B18" s="122" t="n">
-        <v>8.65</v>
+      <c r="B18" s="122">
+        <f>IFERROR(INDEX(Pertes_singulieres_detail!$K$10:$K$40,MATCH("S5",Pertes_singulieres_detail!$A$10:$A$40,0)),0)</f>
+        <v/>
       </c>
       <c r="E18" s="142" t="n"/>
       <c r="F18" s="144" t="n"/>

</xml_diff>

<commit_message>
sync workbook: link Inputs B18 to detailed singular losses
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1800,8 +1800,9 @@
           <t>Coeff_pertes_singulieres_K_total</t>
         </is>
       </c>
-      <c r="B18" s="122" t="n">
-        <v>8.65</v>
+      <c r="B18" s="122">
+        <f>IFERROR(INDEX(Pertes_singulieres_detail!$K$10:$K$40,MATCH("S5",Pertes_singulieres_detail!$A$10:$A$40,0)),0)</f>
+        <v/>
       </c>
       <c r="E18" s="142" t="n"/>
       <c r="F18" s="144" t="n"/>
@@ -5088,14 +5089,14 @@
     <row r="3">
       <c r="A3" s="231" t="inlineStr">
         <is>
-          <t>Configuration consideree: Toiture -&gt; StormBrixx -&gt; regard regulateur -&gt; branche Jellyfish / branche poste pompage.</t>
+          <t>Configuration consideree: StormBrixx -&gt; regard RP-01 (regulateur) -&gt; split vers poste direct et vers DP-01, puis retour DP-01 au poste.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="232" t="inlineStr">
         <is>
-          <t>IMPORTANT: Les K du regulateur et Jellyfish sont provisoires. Remplacer par les pertes de charge constructeur pour le dimensionnement final.</t>
+          <t>IMPORTANT: Les K du regulateur et du separateur dynamique sont provisoires. Remplacer par les pertes constructeur pour le dimensionnement final.</t>
         </is>
       </c>
     </row>
@@ -5204,17 +5205,18 @@
       </c>
       <c r="B10" s="237" t="inlineStr">
         <is>
-          <t>Bassin retention vers RP-01</t>
+          <t>StormBrixx vers regard RP-01 regulateur</t>
         </is>
       </c>
       <c r="C10" s="237" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E10" s="237" t="n">
-        <v>0.029</v>
+      <c r="E10" s="237">
+        <f>MAX(Routing!$F$2:$F$2000)</f>
+        <v/>
       </c>
       <c r="F10" s="238">
         <f>IF(D10&gt;0,PI()*(D10^2)/4,0)</f>
@@ -5249,7 +5251,7 @@
       </c>
       <c r="N10" s="237" t="inlineStr">
         <is>
-          <t>Conduite entree</t>
+          <t>Troncon commun amont</t>
         </is>
       </c>
       <c r="P10" s="235" t="inlineStr">
@@ -5271,7 +5273,7 @@
       </c>
       <c r="B11" s="237" t="inlineStr">
         <is>
-          <t>RP-01 vers regard regulateur</t>
+          <t>RP-01 vers poste de pompage (branche directe)</t>
         </is>
       </c>
       <c r="C11" s="237" t="n">
@@ -5280,8 +5282,9 @@
       <c r="D11" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E11" s="237" t="n">
-        <v>0.029</v>
+      <c r="E11" s="237">
+        <f>MAX(Routing!$Q$2:$Q$2000)</f>
+        <v/>
       </c>
       <c r="F11" s="238">
         <f>IF(D11&gt;0,PI()*(D11^2)/4,0)</f>
@@ -5316,16 +5319,16 @@
       </c>
       <c r="N11" s="237" t="inlineStr">
         <is>
-          <t>Collecteur principal</t>
+          <t>Branche directe vers poste</t>
         </is>
       </c>
       <c r="P11" s="239" t="inlineStr">
         <is>
-          <t>Vers Jellyfish (S1+S2+S3)</t>
+          <t>Chemin direct vers poste (S1+S2)</t>
         </is>
       </c>
       <c r="Q11" s="238">
-        <f>M10+M11+M12</f>
+        <f>M10+M11</f>
         <v/>
       </c>
     </row>
@@ -5337,7 +5340,7 @@
       </c>
       <c r="B12" s="237" t="inlineStr">
         <is>
-          <t>Regard regulateur vers DP-01 (Jellyfish)</t>
+          <t>RP-01 vers DP-01 separateur dynamique</t>
         </is>
       </c>
       <c r="C12" s="237" t="n">
@@ -5346,8 +5349,9 @@
       <c r="D12" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E12" s="237" t="n">
-        <v>0.029</v>
+      <c r="E12" s="237">
+        <f>MAX(Routing!$P$2:$P$2000)</f>
+        <v/>
       </c>
       <c r="F12" s="238">
         <f>IF(D12&gt;0,PI()*(D12^2)/4,0)</f>
@@ -5382,16 +5386,16 @@
       </c>
       <c r="N12" s="237" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Branche derivee vers separateur</t>
         </is>
       </c>
       <c r="P12" s="239" t="inlineStr">
         <is>
-          <t>Vers poste pompage (S1+S2+S4)</t>
+          <t>Chemin via separateur (S1+S3+S4)</t>
         </is>
       </c>
       <c r="Q12" s="238">
-        <f>M10+M11+M13</f>
+        <f>M10+M12+M13</f>
         <v/>
       </c>
     </row>
@@ -5403,17 +5407,18 @@
       </c>
       <c r="B13" s="237" t="inlineStr">
         <is>
-          <t>Regard regulateur vers poste pompage</t>
+          <t>DP-01 vers poste de pompage (retour)</t>
         </is>
       </c>
       <c r="C13" s="237" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="D13" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E13" s="237" t="n">
-        <v>0.164</v>
+      <c r="E13" s="237">
+        <f>MAX(Routing!$R$2:$R$2000)</f>
+        <v/>
       </c>
       <c r="F13" s="238">
         <f>IF(D13&gt;0,PI()*(D13^2)/4,0)</f>
@@ -5448,12 +5453,12 @@
       </c>
       <c r="N13" s="237" t="inlineStr">
         <is>
-          <t>Branche surverse (Q=163.8 L/s)</t>
+          <t>Retour du separateur vers poste</t>
         </is>
       </c>
       <c r="P13" s="239" t="inlineStr">
         <is>
-          <t>Refoulement pompe (S5)</t>
+          <t>Troncon poste vers RP-02 (S5)</t>
         </is>
       </c>
       <c r="Q13" s="238">
@@ -5469,17 +5474,18 @@
       </c>
       <c r="B14" s="237" t="inlineStr">
         <is>
-          <t>Ligne de refoulement poste pompage</t>
+          <t>Poste de pompage vers RP-02 avec clapet</t>
         </is>
       </c>
       <c r="C14" s="237" t="n">
-        <v>31.5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="237" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E14" s="237" t="n">
-        <v>0.039</v>
+        <v>0.3</v>
+      </c>
+      <c r="E14" s="237">
+        <f>MAX(Routing!$M$2:$M$2000)</f>
+        <v/>
       </c>
       <c r="F14" s="238">
         <f>IF(D14&gt;0,PI()*(D14^2)/4,0)</f>
@@ -5514,12 +5520,12 @@
       </c>
       <c r="N14" s="237" t="inlineStr">
         <is>
-          <t>Refoulement pompe (Q unitaire)</t>
+          <t>Aval poste vers RP-02</t>
         </is>
       </c>
       <c r="P14" s="239" t="inlineStr">
         <is>
-          <t>Exutoire gravitaire aval (S6)</t>
+          <t>Troncon aval gravitaire (S6)</t>
         </is>
       </c>
       <c r="Q14" s="238">
@@ -5535,17 +5541,18 @@
       </c>
       <c r="B15" s="237" t="inlineStr">
         <is>
-          <t>RP avec clapet vers exutoire gravite</t>
+          <t>RP-02 vers exutoire gravitaire</t>
         </is>
       </c>
       <c r="C15" s="237" t="n">
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="D15" s="237" t="n">
         <v>0.3</v>
       </c>
-      <c r="E15" s="237" t="n">
-        <v>0.039</v>
+      <c r="E15" s="237">
+        <f>E14</f>
+        <v/>
       </c>
       <c r="F15" s="238">
         <f>IF(D15&gt;0,PI()*(D15^2)/4,0)</f>
@@ -5580,7 +5587,7 @@
       </c>
       <c r="N15" s="237" t="inlineStr">
         <is>
-          <t>Troncon aval gravitaire</t>
+          <t>Troncon final a gravite</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5599,7 @@
       </c>
       <c r="Q17" s="116" t="inlineStr">
         <is>
-          <t>Valider K Jellyfish et K regulateur sur fiches fabricants.</t>
+          <t>Valider K regulateur, K separateur et K clapet RP-02 sur fiches fabricants.</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5645,7 @@
       </c>
       <c r="B21" s="237" t="inlineStr">
         <is>
-          <t>Entree brusque</t>
+          <t>Entree depuis StormBrixx</t>
         </is>
       </c>
       <c r="C21" s="237" t="n">
@@ -5660,14 +5667,14 @@
       </c>
       <c r="B22" s="237" t="inlineStr">
         <is>
-          <t>Coude 90 rayon court</t>
+          <t>Regard RP-01 (passage)</t>
         </is>
       </c>
       <c r="C22" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="237" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="238">
         <f>C22*D22</f>
@@ -5677,19 +5684,19 @@
     <row r="23">
       <c r="A23" s="237" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B23" s="237" t="inlineStr">
         <is>
-          <t>Regard traversant</t>
+          <t>Regulateur RP-01 (provisoire)</t>
         </is>
       </c>
       <c r="C23" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="237" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="E23" s="238">
         <f>C23*D23</f>
@@ -5704,14 +5711,14 @@
       </c>
       <c r="B24" s="237" t="inlineStr">
         <is>
-          <t>Coude 45</t>
+          <t>Te passage droit (vers branche directe)</t>
         </is>
       </c>
       <c r="C24" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="237" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E24" s="238">
         <f>C24*D24</f>
@@ -5721,19 +5728,19 @@
     <row r="25">
       <c r="A25" s="237" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B25" s="237" t="inlineStr">
         <is>
-          <t>Te derivation</t>
+          <t>Coude de raccordement vers poste</t>
         </is>
       </c>
       <c r="C25" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="237" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="E25" s="238">
         <f>C25*D25</f>
@@ -5748,14 +5755,14 @@
       </c>
       <c r="B26" s="237" t="inlineStr">
         <is>
-          <t>Equipement Jellyfish (provisoire)</t>
+          <t>Te derivation vers DP-01</t>
         </is>
       </c>
       <c r="C26" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="237" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E26" s="238">
         <f>C26*D26</f>
@@ -5765,19 +5772,19 @@
     <row r="27">
       <c r="A27" s="237" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B27" s="237" t="inlineStr">
         <is>
-          <t>Te passage droit</t>
+          <t>Entree separateur dynamique</t>
         </is>
       </c>
       <c r="C27" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="237" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="238">
         <f>C27*D27</f>
@@ -5792,14 +5799,14 @@
       </c>
       <c r="B28" s="237" t="inlineStr">
         <is>
-          <t>Regulateur Q-brake (provisoire)</t>
+          <t>Sortie separateur dynamique (provisoire)</t>
         </is>
       </c>
       <c r="C28" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="237" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E28" s="238">
         <f>C28*D28</f>
@@ -5809,19 +5816,19 @@
     <row r="29">
       <c r="A29" s="237" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B29" s="237" t="inlineStr">
         <is>
-          <t>Clapet anti-retour</t>
+          <t>Raccord retour vers poste</t>
         </is>
       </c>
       <c r="C29" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="237" t="n">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="E29" s="238">
         <f>C29*D29</f>
@@ -5836,14 +5843,14 @@
       </c>
       <c r="B30" s="237" t="inlineStr">
         <is>
-          <t>Vanne d'isolement ouverte</t>
+          <t>Clapet anti-retour RP-02</t>
         </is>
       </c>
       <c r="C30" s="237" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="237" t="n">
-        <v>0.2</v>
+        <v>2.5</v>
       </c>
       <c r="E30" s="238">
         <f>C30*D30</f>
@@ -5858,11 +5865,11 @@
       </c>
       <c r="B31" s="237" t="inlineStr">
         <is>
-          <t>Coude 90 (x2)</t>
+          <t>Coude 90</t>
         </is>
       </c>
       <c r="C31" s="237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="237" t="n">
         <v>0.9</v>
@@ -5880,7 +5887,7 @@
       </c>
       <c r="B32" s="237" t="inlineStr">
         <is>
-          <t>Sortie libre</t>
+          <t>Sortie libre a l'exutoire</t>
         </is>
       </c>
       <c r="C32" s="237" t="n">

</xml_diff>

<commit_message>
Fix BlockDepth lookup N/A for odd hyetograph steps
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -2449,7 +2449,7 @@
         <v/>
       </c>
       <c r="F2" s="166">
-        <f>IF(E2="","",IF(E2=1,Inputs!$B$53/2,IF(MOD(E2,2)=0,Inputs!$B$53/2+E2/2,Inputs!$B$53/2-(E2-1)/2)))</f>
+        <f>IF(E2="","",IF(E2=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E2,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E2/2,ROUNDUP(Inputs!$B$53/2,0)-(E2-1)/2)))</f>
         <v/>
       </c>
       <c r="H2" s="116" t="n">
@@ -2490,7 +2490,7 @@
         <v/>
       </c>
       <c r="F3" s="166">
-        <f>IF(E3="","",IF(E3=1,Inputs!$B$53/2,IF(MOD(E3,2)=0,Inputs!$B$53/2+E3/2,Inputs!$B$53/2-(E3-1)/2)))</f>
+        <f>IF(E3="","",IF(E3=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E3,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E3/2,ROUNDUP(Inputs!$B$53/2,0)-(E3-1)/2)))</f>
         <v/>
       </c>
       <c r="H3" s="116" t="n">
@@ -2531,7 +2531,7 @@
         <v/>
       </c>
       <c r="F4" s="166">
-        <f>IF(E4="","",IF(E4=1,Inputs!$B$53/2,IF(MOD(E4,2)=0,Inputs!$B$53/2+E4/2,Inputs!$B$53/2-(E4-1)/2)))</f>
+        <f>IF(E4="","",IF(E4=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E4,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E4/2,ROUNDUP(Inputs!$B$53/2,0)-(E4-1)/2)))</f>
         <v/>
       </c>
       <c r="H4" s="116" t="n">
@@ -2572,7 +2572,7 @@
         <v/>
       </c>
       <c r="F5" s="166">
-        <f>IF(E5="","",IF(E5=1,Inputs!$B$53/2,IF(MOD(E5,2)=0,Inputs!$B$53/2+E5/2,Inputs!$B$53/2-(E5-1)/2)))</f>
+        <f>IF(E5="","",IF(E5=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E5,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E5/2,ROUNDUP(Inputs!$B$53/2,0)-(E5-1)/2)))</f>
         <v/>
       </c>
       <c r="H5" s="116" t="n">
@@ -2613,7 +2613,7 @@
         <v/>
       </c>
       <c r="F6" s="166">
-        <f>IF(E6="","",IF(E6=1,Inputs!$B$53/2,IF(MOD(E6,2)=0,Inputs!$B$53/2+E6/2,Inputs!$B$53/2-(E6-1)/2)))</f>
+        <f>IF(E6="","",IF(E6=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E6,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E6/2,ROUNDUP(Inputs!$B$53/2,0)-(E6-1)/2)))</f>
         <v/>
       </c>
       <c r="H6" s="116" t="n">
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="F7" s="166">
-        <f>IF(E7="","",IF(E7=1,Inputs!$B$53/2,IF(MOD(E7,2)=0,Inputs!$B$53/2+E7/2,Inputs!$B$53/2-(E7-1)/2)))</f>
+        <f>IF(E7="","",IF(E7=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E7,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E7/2,ROUNDUP(Inputs!$B$53/2,0)-(E7-1)/2)))</f>
         <v/>
       </c>
       <c r="H7" s="116" t="n">
@@ -2695,7 +2695,7 @@
         <v/>
       </c>
       <c r="F8" s="166">
-        <f>IF(E8="","",IF(E8=1,Inputs!$B$53/2,IF(MOD(E8,2)=0,Inputs!$B$53/2+E8/2,Inputs!$B$53/2-(E8-1)/2)))</f>
+        <f>IF(E8="","",IF(E8=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E8,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E8/2,ROUNDUP(Inputs!$B$53/2,0)-(E8-1)/2)))</f>
         <v/>
       </c>
       <c r="H8" s="116" t="n">
@@ -2736,7 +2736,7 @@
         <v/>
       </c>
       <c r="F9" s="166">
-        <f>IF(E9="","",IF(E9=1,Inputs!$B$53/2,IF(MOD(E9,2)=0,Inputs!$B$53/2+E9/2,Inputs!$B$53/2-(E9-1)/2)))</f>
+        <f>IF(E9="","",IF(E9=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E9,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E9/2,ROUNDUP(Inputs!$B$53/2,0)-(E9-1)/2)))</f>
         <v/>
       </c>
       <c r="H9" s="116" t="n">
@@ -2777,7 +2777,7 @@
         <v/>
       </c>
       <c r="F10" s="166">
-        <f>IF(E10="","",IF(E10=1,Inputs!$B$53/2,IF(MOD(E10,2)=0,Inputs!$B$53/2+E10/2,Inputs!$B$53/2-(E10-1)/2)))</f>
+        <f>IF(E10="","",IF(E10=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E10,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E10/2,ROUNDUP(Inputs!$B$53/2,0)-(E10-1)/2)))</f>
         <v/>
       </c>
       <c r="H10" s="116" t="n">
@@ -2818,7 +2818,7 @@
         <v/>
       </c>
       <c r="F11" s="166">
-        <f>IF(E11="","",IF(E11=1,Inputs!$B$53/2,IF(MOD(E11,2)=0,Inputs!$B$53/2+E11/2,Inputs!$B$53/2-(E11-1)/2)))</f>
+        <f>IF(E11="","",IF(E11=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E11,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E11/2,ROUNDUP(Inputs!$B$53/2,0)-(E11-1)/2)))</f>
         <v/>
       </c>
       <c r="H11" s="116" t="n">
@@ -2859,7 +2859,7 @@
         <v/>
       </c>
       <c r="F12" s="166">
-        <f>IF(E12="","",IF(E12=1,Inputs!$B$53/2,IF(MOD(E12,2)=0,Inputs!$B$53/2+E12/2,Inputs!$B$53/2-(E12-1)/2)))</f>
+        <f>IF(E12="","",IF(E12=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E12,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E12/2,ROUNDUP(Inputs!$B$53/2,0)-(E12-1)/2)))</f>
         <v/>
       </c>
       <c r="H12" s="116" t="n">
@@ -2900,7 +2900,7 @@
         <v/>
       </c>
       <c r="F13" s="166">
-        <f>IF(E13="","",IF(E13=1,Inputs!$B$53/2,IF(MOD(E13,2)=0,Inputs!$B$53/2+E13/2,Inputs!$B$53/2-(E13-1)/2)))</f>
+        <f>IF(E13="","",IF(E13=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E13,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E13/2,ROUNDUP(Inputs!$B$53/2,0)-(E13-1)/2)))</f>
         <v/>
       </c>
       <c r="H13" s="116" t="n">
@@ -2941,7 +2941,7 @@
         <v/>
       </c>
       <c r="F14" s="163">
-        <f>IF(E14="","",IF(E14=1,Inputs!$B$53/2,IF(MOD(E14,2)=0,Inputs!$B$53/2+E14/2,Inputs!$B$53/2-(E14-1)/2)))</f>
+        <f>IF(E14="","",IF(E14=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E14,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E14/2,ROUNDUP(Inputs!$B$53/2,0)-(E14-1)/2)))</f>
         <v/>
       </c>
       <c r="H14" s="116" t="n">
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="F15" s="163">
-        <f>IF(E15="","",IF(E15=1,Inputs!$B$53/2,IF(MOD(E15,2)=0,Inputs!$B$53/2+E15/2,Inputs!$B$53/2-(E15-1)/2)))</f>
+        <f>IF(E15="","",IF(E15=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E15,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E15/2,ROUNDUP(Inputs!$B$53/2,0)-(E15-1)/2)))</f>
         <v/>
       </c>
       <c r="H15" s="116" t="n">
@@ -3023,7 +3023,7 @@
         <v/>
       </c>
       <c r="F16" s="116">
-        <f>IF(E16="","",IF(E16=1,Inputs!$B$53/2,IF(MOD(E16,2)=0,Inputs!$B$53/2+E16/2,Inputs!$B$53/2-(E16-1)/2)))</f>
+        <f>IF(E16="","",IF(E16=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E16,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E16/2,ROUNDUP(Inputs!$B$53/2,0)-(E16-1)/2)))</f>
         <v/>
       </c>
       <c r="H16" s="116" t="n">
@@ -3064,7 +3064,7 @@
         <v/>
       </c>
       <c r="F17" s="116">
-        <f>IF(E17="","",IF(E17=1,Inputs!$B$53/2,IF(MOD(E17,2)=0,Inputs!$B$53/2+E17/2,Inputs!$B$53/2-(E17-1)/2)))</f>
+        <f>IF(E17="","",IF(E17=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E17,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E17/2,ROUNDUP(Inputs!$B$53/2,0)-(E17-1)/2)))</f>
         <v/>
       </c>
       <c r="H17" s="116" t="n">
@@ -3105,7 +3105,7 @@
         <v/>
       </c>
       <c r="F18" s="116">
-        <f>IF(E18="","",IF(E18=1,Inputs!$B$53/2,IF(MOD(E18,2)=0,Inputs!$B$53/2+E18/2,Inputs!$B$53/2-(E18-1)/2)))</f>
+        <f>IF(E18="","",IF(E18=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E18,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E18/2,ROUNDUP(Inputs!$B$53/2,0)-(E18-1)/2)))</f>
         <v/>
       </c>
       <c r="H18" s="116" t="n">
@@ -3146,7 +3146,7 @@
         <v/>
       </c>
       <c r="F19" s="116">
-        <f>IF(E19="","",IF(E19=1,Inputs!$B$53/2,IF(MOD(E19,2)=0,Inputs!$B$53/2+E19/2,Inputs!$B$53/2-(E19-1)/2)))</f>
+        <f>IF(E19="","",IF(E19=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E19,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E19/2,ROUNDUP(Inputs!$B$53/2,0)-(E19-1)/2)))</f>
         <v/>
       </c>
       <c r="H19" s="116" t="n">
@@ -3187,7 +3187,7 @@
         <v/>
       </c>
       <c r="F20" s="116">
-        <f>IF(E20="","",IF(E20=1,Inputs!$B$53/2,IF(MOD(E20,2)=0,Inputs!$B$53/2+E20/2,Inputs!$B$53/2-(E20-1)/2)))</f>
+        <f>IF(E20="","",IF(E20=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E20,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E20/2,ROUNDUP(Inputs!$B$53/2,0)-(E20-1)/2)))</f>
         <v/>
       </c>
       <c r="H20" s="116" t="n">
@@ -3228,7 +3228,7 @@
         <v/>
       </c>
       <c r="F21" s="116">
-        <f>IF(E21="","",IF(E21=1,Inputs!$B$53/2,IF(MOD(E21,2)=0,Inputs!$B$53/2+E21/2,Inputs!$B$53/2-(E21-1)/2)))</f>
+        <f>IF(E21="","",IF(E21=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E21,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E21/2,ROUNDUP(Inputs!$B$53/2,0)-(E21-1)/2)))</f>
         <v/>
       </c>
       <c r="H21" s="116" t="n">
@@ -3269,7 +3269,7 @@
         <v/>
       </c>
       <c r="F22" s="116">
-        <f>IF(E22="","",IF(E22=1,Inputs!$B$53/2,IF(MOD(E22,2)=0,Inputs!$B$53/2+E22/2,Inputs!$B$53/2-(E22-1)/2)))</f>
+        <f>IF(E22="","",IF(E22=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E22,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E22/2,ROUNDUP(Inputs!$B$53/2,0)-(E22-1)/2)))</f>
         <v/>
       </c>
       <c r="H22" s="116" t="n">
@@ -3310,7 +3310,7 @@
         <v/>
       </c>
       <c r="F23" s="116">
-        <f>IF(E23="","",IF(E23=1,Inputs!$B$53/2,IF(MOD(E23,2)=0,Inputs!$B$53/2+E23/2,Inputs!$B$53/2-(E23-1)/2)))</f>
+        <f>IF(E23="","",IF(E23=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E23,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E23/2,ROUNDUP(Inputs!$B$53/2,0)-(E23-1)/2)))</f>
         <v/>
       </c>
       <c r="H23" s="116" t="n">
@@ -3351,7 +3351,7 @@
         <v/>
       </c>
       <c r="F24" s="116">
-        <f>IF(E24="","",IF(E24=1,Inputs!$B$53/2,IF(MOD(E24,2)=0,Inputs!$B$53/2+E24/2,Inputs!$B$53/2-(E24-1)/2)))</f>
+        <f>IF(E24="","",IF(E24=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E24,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E24/2,ROUNDUP(Inputs!$B$53/2,0)-(E24-1)/2)))</f>
         <v/>
       </c>
       <c r="H24" s="116" t="n">
@@ -3392,7 +3392,7 @@
         <v/>
       </c>
       <c r="F25" s="116">
-        <f>IF(E25="","",IF(E25=1,Inputs!$B$53/2,IF(MOD(E25,2)=0,Inputs!$B$53/2+E25/2,Inputs!$B$53/2-(E25-1)/2)))</f>
+        <f>IF(E25="","",IF(E25=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E25,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E25/2,ROUNDUP(Inputs!$B$53/2,0)-(E25-1)/2)))</f>
         <v/>
       </c>
       <c r="H25" s="116" t="n">
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="F26" s="116">
-        <f>IF(E26="","",IF(E26=1,Inputs!$B$53/2,IF(MOD(E26,2)=0,Inputs!$B$53/2+E26/2,Inputs!$B$53/2-(E26-1)/2)))</f>
+        <f>IF(E26="","",IF(E26=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E26,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E26/2,ROUNDUP(Inputs!$B$53/2,0)-(E26-1)/2)))</f>
         <v/>
       </c>
       <c r="H26" s="116" t="n">
@@ -3474,7 +3474,7 @@
         <v/>
       </c>
       <c r="F27" s="116">
-        <f>IF(E27="","",IF(E27=1,Inputs!$B$53/2,IF(MOD(E27,2)=0,Inputs!$B$53/2+E27/2,Inputs!$B$53/2-(E27-1)/2)))</f>
+        <f>IF(E27="","",IF(E27=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E27,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E27/2,ROUNDUP(Inputs!$B$53/2,0)-(E27-1)/2)))</f>
         <v/>
       </c>
       <c r="H27" s="116" t="n">
@@ -3515,7 +3515,7 @@
         <v/>
       </c>
       <c r="F28" s="116">
-        <f>IF(E28="","",IF(E28=1,Inputs!$B$53/2,IF(MOD(E28,2)=0,Inputs!$B$53/2+E28/2,Inputs!$B$53/2-(E28-1)/2)))</f>
+        <f>IF(E28="","",IF(E28=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E28,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E28/2,ROUNDUP(Inputs!$B$53/2,0)-(E28-1)/2)))</f>
         <v/>
       </c>
       <c r="H28" s="116" t="n">
@@ -3556,7 +3556,7 @@
         <v/>
       </c>
       <c r="F29" s="116">
-        <f>IF(E29="","",IF(E29=1,Inputs!$B$53/2,IF(MOD(E29,2)=0,Inputs!$B$53/2+E29/2,Inputs!$B$53/2-(E29-1)/2)))</f>
+        <f>IF(E29="","",IF(E29=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E29,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E29/2,ROUNDUP(Inputs!$B$53/2,0)-(E29-1)/2)))</f>
         <v/>
       </c>
       <c r="H29" s="116" t="n">
@@ -3597,7 +3597,7 @@
         <v/>
       </c>
       <c r="F30" s="116">
-        <f>IF(E30="","",IF(E30=1,Inputs!$B$53/2,IF(MOD(E30,2)=0,Inputs!$B$53/2+E30/2,Inputs!$B$53/2-(E30-1)/2)))</f>
+        <f>IF(E30="","",IF(E30=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E30,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E30/2,ROUNDUP(Inputs!$B$53/2,0)-(E30-1)/2)))</f>
         <v/>
       </c>
       <c r="H30" s="116" t="n">
@@ -3638,7 +3638,7 @@
         <v/>
       </c>
       <c r="F31" s="116">
-        <f>IF(E31="","",IF(E31=1,Inputs!$B$53/2,IF(MOD(E31,2)=0,Inputs!$B$53/2+E31/2,Inputs!$B$53/2-(E31-1)/2)))</f>
+        <f>IF(E31="","",IF(E31=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E31,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E31/2,ROUNDUP(Inputs!$B$53/2,0)-(E31-1)/2)))</f>
         <v/>
       </c>
       <c r="H31" s="116" t="n">
@@ -3679,7 +3679,7 @@
         <v/>
       </c>
       <c r="F32" s="116">
-        <f>IF(E32="","",IF(E32=1,Inputs!$B$53/2,IF(MOD(E32,2)=0,Inputs!$B$53/2+E32/2,Inputs!$B$53/2-(E32-1)/2)))</f>
+        <f>IF(E32="","",IF(E32=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E32,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E32/2,ROUNDUP(Inputs!$B$53/2,0)-(E32-1)/2)))</f>
         <v/>
       </c>
       <c r="H32" s="116" t="n">
@@ -3720,7 +3720,7 @@
         <v/>
       </c>
       <c r="F33" s="116">
-        <f>IF(E33="","",IF(E33=1,Inputs!$B$53/2,IF(MOD(E33,2)=0,Inputs!$B$53/2+E33/2,Inputs!$B$53/2-(E33-1)/2)))</f>
+        <f>IF(E33="","",IF(E33=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E33,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E33/2,ROUNDUP(Inputs!$B$53/2,0)-(E33-1)/2)))</f>
         <v/>
       </c>
       <c r="H33" s="116" t="n">
@@ -3761,7 +3761,7 @@
         <v/>
       </c>
       <c r="F34" s="116">
-        <f>IF(E34="","",IF(E34=1,Inputs!$B$53/2,IF(MOD(E34,2)=0,Inputs!$B$53/2+E34/2,Inputs!$B$53/2-(E34-1)/2)))</f>
+        <f>IF(E34="","",IF(E34=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E34,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E34/2,ROUNDUP(Inputs!$B$53/2,0)-(E34-1)/2)))</f>
         <v/>
       </c>
       <c r="H34" s="116" t="n">
@@ -3802,7 +3802,7 @@
         <v/>
       </c>
       <c r="F35" s="116">
-        <f>IF(E35="","",IF(E35=1,Inputs!$B$53/2,IF(MOD(E35,2)=0,Inputs!$B$53/2+E35/2,Inputs!$B$53/2-(E35-1)/2)))</f>
+        <f>IF(E35="","",IF(E35=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E35,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E35/2,ROUNDUP(Inputs!$B$53/2,0)-(E35-1)/2)))</f>
         <v/>
       </c>
       <c r="H35" s="116" t="n">
@@ -3843,7 +3843,7 @@
         <v/>
       </c>
       <c r="F36" s="116">
-        <f>IF(E36="","",IF(E36=1,Inputs!$B$53/2,IF(MOD(E36,2)=0,Inputs!$B$53/2+E36/2,Inputs!$B$53/2-(E36-1)/2)))</f>
+        <f>IF(E36="","",IF(E36=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E36,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E36/2,ROUNDUP(Inputs!$B$53/2,0)-(E36-1)/2)))</f>
         <v/>
       </c>
       <c r="H36" s="116" t="n">
@@ -3884,7 +3884,7 @@
         <v/>
       </c>
       <c r="F37" s="116">
-        <f>IF(E37="","",IF(E37=1,Inputs!$B$53/2,IF(MOD(E37,2)=0,Inputs!$B$53/2+E37/2,Inputs!$B$53/2-(E37-1)/2)))</f>
+        <f>IF(E37="","",IF(E37=1,ROUNDUP(Inputs!$B$53/2,0),IF(MOD(E37,2)=0,ROUNDUP(Inputs!$B$53/2,0)+E37/2,ROUNDUP(Inputs!$B$53/2,0)-(E37-1)/2)))</f>
         <v/>
       </c>
       <c r="H37" s="116" t="n">
@@ -4110,7 +4110,7 @@
         <v>1</v>
       </c>
       <c r="V2" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U2, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U2, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
         <v>2</v>
       </c>
       <c r="V3" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U3, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U3, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
         <v>3</v>
       </c>
       <c r="V4" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U4, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U4, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
         <v>4</v>
       </c>
       <c r="V5" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U5, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U5, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
         <v>5</v>
       </c>
       <c r="V6" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U6, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U6, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
         <v>6</v>
       </c>
       <c r="V7" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U7, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U7, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
         <v>7</v>
       </c>
       <c r="V8" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U8, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U8, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
         <v>8</v>
       </c>
       <c r="V9" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U9, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U9, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
         <v>9</v>
       </c>
       <c r="V10" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U10, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U10, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
         <v>10</v>
       </c>
       <c r="V11" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U11, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U11, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
         <v>11</v>
       </c>
       <c r="V12" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U12, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U12, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
         <v>12</v>
       </c>
       <c r="V13" s="165">
-        <f>INDEX(IDF_Hyetograph!$D$2:$D$13, MATCH(U13, IDF_Hyetograph!$F$2:$F$13, 0))</f>
+        <f>IFERROR(INDEX(IDF_Hyetograph!$D$2:$D$37, MATCH(U13, IDF_Hyetograph!$F$2:$F$37, 0)),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Link wetwell depth to top level minus invert
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -2161,8 +2161,25 @@
       <c r="B38" s="122" t="n"/>
     </row>
     <row r="39" ht="12.75" customHeight="1" s="117">
-      <c r="A39" s="121" t="n"/>
-      <c r="B39" s="122" t="n"/>
+      <c r="A39" s="121" t="inlineStr">
+        <is>
+          <t>Wetwell_top_level_m</t>
+        </is>
+      </c>
+      <c r="B39" s="242">
+        <f>MAX(B45,B46)+0.30</f>
+        <v/>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Niveau de référence du puits (couvercle/limite utile). Ajustable. Par défaut: max niveau marche/arrêt + 0.30 m.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="12.75" customHeight="1" s="117">
       <c r="A40" s="156" t="inlineStr">
@@ -2213,14 +2230,19 @@
           <t>Wetwell_total_depth_m</t>
         </is>
       </c>
-      <c r="B43" s="242" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="C43" s="116" t="n">
-        <v>3</v>
-      </c>
-      <c r="D43" s="116" t="n">
-        <v>2</v>
+      <c r="B43" s="242">
+        <f>MAX(0,B39-B40)</f>
+        <v/>
+      </c>
+      <c r="C43" s="116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D43" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur utile calculée = Wetwell_top_level_m - Wetwell_invert_m.</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="12.75" customHeight="1" s="117">

</xml_diff>

<commit_message>
Add compact foundation drain flow calculator in Inputs
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23.48" customWidth="1" style="116" min="1" max="1"/>
@@ -2365,6 +2365,88 @@
       <c r="B53" s="251">
         <f>ROUNDUP(B52/B8,0)</f>
         <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="160" t="inlineStr">
+        <is>
+          <t>Foundation_drain_length_m</t>
+        </is>
+      </c>
+      <c r="B55" s="249" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Longueur active de drains de fondation raccordes au bassin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="160" t="inlineStr">
+        <is>
+          <t>Foundation_drain_unit_flow_Ls_per_100m</t>
+        </is>
+      </c>
+      <c r="B56" s="249" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>L/s/100m</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Debit unitaire preliminaire (a calibrer avec donnees terrain/saison humide).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_drain_m3s</t>
+        </is>
+      </c>
+      <c r="B57" s="249">
+        <f>B55*B56/100/1000</f>
+        <v/>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Debit constant equivalent a ajouter manuellement aux scenarios de verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="160" t="inlineStr">
+        <is>
+          <t>V_foundation_drain_event_m3</t>
+        </is>
+      </c>
+      <c r="B58" s="249">
+        <f>B57*B52*60</f>
+        <v/>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Volume genere pendant la duree d evenement (Inputs!B52).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -21895,7 +21977,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="116" t="inlineStr">
         <is>
           <t>Invert_regard_aval_m</t>
         </is>
@@ -21903,17 +21985,17 @@
       <c r="B5" s="282" t="n">
         <v>103.03</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="116" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="116" t="inlineStr">
         <is>
           <t>Fond du regard aval</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="116" t="inlineStr">
         <is>
           <t>Vmax_calcule_m3</t>
         </is>
@@ -21934,7 +22016,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="116" t="inlineStr">
         <is>
           <t>Diametre_regard_aval_m</t>
         </is>
@@ -21942,17 +22024,17 @@
       <c r="B6" s="282" t="n">
         <v>1.5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="116" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="116" t="inlineStr">
         <is>
           <t>Diametre interieur utile</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="116" t="inlineStr">
         <is>
           <t>Vreq_avec_FS_m3</t>
         </is>
@@ -21970,7 +22052,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="116" t="inlineStr">
         <is>
           <t>Aire_regard_aval_m2</t>
         </is>
@@ -21979,17 +22061,17 @@
         <f>PI()*B6^2/4</f>
         <v/>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="116" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="116" t="inlineStr">
         <is>
           <t>Aire de stockage verticale</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="116" t="inlineStr">
         <is>
           <t>Hauteur_req_m</t>
         </is>
@@ -22007,7 +22089,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="116" t="inlineStr">
         <is>
           <t>Volume_initial_m3</t>
         </is>
@@ -22015,17 +22097,17 @@
       <c r="B8" s="282" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="116" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="116" t="inlineStr">
         <is>
           <t>Condition initiale au debut de l evenement</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="116" t="inlineStr">
         <is>
           <t>Niveau_eau_max_requis_m</t>
         </is>
@@ -22043,7 +22125,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="116" t="inlineStr">
         <is>
           <t>Facteur_securite_stockage</t>
         </is>
@@ -22051,17 +22133,17 @@
       <c r="B9" s="282" t="n">
         <v>1.15</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="116" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="116" t="inlineStr">
         <is>
           <t>Applique sur Vmax</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="116" t="inlineStr">
         <is>
           <t>Verification_niveau</t>
         </is>
@@ -22079,7 +22161,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="116" t="inlineStr">
         <is>
           <t>Pas_temps_sec</t>
         </is>
@@ -22088,17 +22170,17 @@
         <f>Inputs!$B$9</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="116" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="116" t="inlineStr">
         <is>
           <t>Pas du routage (doit suivre Inputs)</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="116" t="inlineStr">
         <is>
           <t>Marge_niveau_m</t>
         </is>
@@ -22116,7 +22198,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="116" t="inlineStr">
         <is>
           <t>Nb_pas_evenement</t>
         </is>
@@ -22125,12 +22207,12 @@
         <f>Inputs!$B$53</f>
         <v/>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="116" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="116" t="inlineStr">
         <is>
           <t>Nombre de pas actifs depuis Inputs</t>
         </is>
@@ -22144,7 +22226,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="116" t="inlineStr">
         <is>
           <t>Niveau_max_admissible_m</t>
         </is>
@@ -22153,17 +22235,17 @@
         <f>B5+1.00</f>
         <v/>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="116" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="116" t="inlineStr">
         <is>
           <t>Ajuster selon geometre/rim/freeboard</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="116" t="inlineStr">
         <is>
           <t>Note: Niveaux J6:J11 doivent etre croissants.</t>
         </is>

</xml_diff>

<commit_message>
Add foundation drain toggle and what-if pumping margin block
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23.48" customWidth="1" style="116" min="1" max="1"/>
@@ -2376,12 +2376,12 @@
       <c r="B55" s="249" t="n">
         <v>0</v>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="116" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="116" t="inlineStr">
         <is>
           <t>Longueur active de drains de fondation raccordes au bassin.</t>
         </is>
@@ -2396,12 +2396,12 @@
       <c r="B56" s="249" t="n">
         <v>0.8</v>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="116" t="inlineStr">
         <is>
           <t>L/s/100m</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="116" t="inlineStr">
         <is>
           <t>Debit unitaire preliminaire (a calibrer avec donnees terrain/saison humide).</t>
         </is>
@@ -2417,12 +2417,12 @@
         <f>B55*B56/100/1000</f>
         <v/>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="116" t="inlineStr">
         <is>
           <t>m3/s</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="116" t="inlineStr">
         <is>
           <t>Debit constant equivalent a ajouter manuellement aux scenarios de verification.</t>
         </is>
@@ -2438,14 +2438,183 @@
         <f>B57*B52*60</f>
         <v/>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="116" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="116" t="inlineStr">
         <is>
           <t>Volume genere pendant la duree d evenement (Inputs!B52).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="160" t="inlineStr">
+        <is>
+          <t>Include_foundation_drain_in_whatif</t>
+        </is>
+      </c>
+      <c r="B59" s="249" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C59" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="116" t="inlineStr">
+        <is>
+          <t>YES/OUI pour inclure le debit de drains de fondation dans le calcul what-if (sans changer la logique principale).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_drain_used_m3s</t>
+        </is>
+      </c>
+      <c r="B60" s="249">
+        <f>IF(OR(UPPER(TRIM(B59))="YES",UPPER(TRIM(B59))="OUI",UPPER(TRIM(B59))="Y"),B57,0)</f>
+        <v/>
+      </c>
+      <c r="C60" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D60" s="116" t="inlineStr">
+        <is>
+          <t>Debit de drains effectivement retenu selon le toggle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="160" t="inlineStr">
+        <is>
+          <t>V_foundation_drain_used_event_m3</t>
+        </is>
+      </c>
+      <c r="B61" s="249">
+        <f>B60*B52*60</f>
+        <v/>
+      </c>
+      <c r="C61" s="116" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D61" s="116" t="inlineStr">
+        <is>
+          <t>Volume additionnel pendant la duree d evenement (what-if).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="160" t="inlineStr">
+        <is>
+          <t>Q_peak_base_proxy_m3s</t>
+        </is>
+      </c>
+      <c r="B62" s="249">
+        <f>IFERROR(INDEX(Analyse_duree!$E$5:$E$8,MATCH(B52,Analyse_duree!$A$5:$A$8,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C62" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D62" s="116" t="inlineStr">
+        <is>
+          <t>Debit de pointe proxy de base (sans drains de fondation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="160" t="inlineStr">
+        <is>
+          <t>Q_peak_whatif_with_foundation_m3s</t>
+        </is>
+      </c>
+      <c r="B63" s="249">
+        <f>IF(B62="","",B62+B60)</f>
+        <v/>
+      </c>
+      <c r="C63" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D63" s="116" t="inlineStr">
+        <is>
+          <t>Debit de pointe what-if = base + drains de fondation inclus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="160" t="inlineStr">
+        <is>
+          <t>Q_pumping_total_capacity_m3s</t>
+        </is>
+      </c>
+      <c r="B64" s="249">
+        <f>B13*B14</f>
+        <v/>
+      </c>
+      <c r="C64" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D64" s="116" t="inlineStr">
+        <is>
+          <t>Capacite de pompage installee (debit unitaire x nb pompes en service).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="160" t="inlineStr">
+        <is>
+          <t>Q_margin_pumping_minus_whatif_m3s</t>
+        </is>
+      </c>
+      <c r="B65" s="249">
+        <f>IF(OR(B63="",B64=""),"",B64-B63)</f>
+        <v/>
+      </c>
+      <c r="C65" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D65" s="116" t="inlineStr">
+        <is>
+          <t>Marge positive = capacite suffisante au pic what-if.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="160" t="inlineStr">
+        <is>
+          <t>Whatif_status_foundation_vs_pumping</t>
+        </is>
+      </c>
+      <c r="B66" s="249">
+        <f>IF(B65="","INFO",IF(B65&gt;=0,"OK","DEFICIT"))</f>
+        <v/>
+      </c>
+      <c r="C66" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D66" s="116" t="inlineStr">
+        <is>
+          <t>Indicateur rapide de risque si drains de fondation sont ajoutes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add QUICK/DARCY method selector with low-base-high scenarios
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -517,7 +517,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="290">
+  <cellXfs count="292">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1340,6 +1340,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="11" fontId="8" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1569,7 +1575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23.48" customWidth="1" style="116" min="1" max="1"/>
@@ -2478,7 +2484,7 @@
         </is>
       </c>
       <c r="B60" s="249">
-        <f>IF(OR(UPPER(TRIM(B59))="YES",UPPER(TRIM(B59))="OUI",UPPER(TRIM(B59))="Y"),B57,0)</f>
+        <f>IF(OR(UPPER(TRIM(B59))="YES",UPPER(TRIM(B59))="OUI",UPPER(TRIM(B59))="Y"),B85,0)</f>
         <v/>
       </c>
       <c r="C60" s="116" t="inlineStr">
@@ -2488,7 +2494,7 @@
       </c>
       <c r="D60" s="116" t="inlineStr">
         <is>
-          <t>Debit de drains effectivement retenu selon le toggle.</t>
+          <t>Debit de drains effectivement retenu selon toggle et methode selectionnee (QUICK/DARCY).</t>
         </is>
       </c>
     </row>
@@ -2615,6 +2621,416 @@
       <c r="D66" s="116" t="inlineStr">
         <is>
           <t>Indicateur rapide de risque si drains de fondation sont ajoutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="160" t="inlineStr">
+        <is>
+          <t>Foundation_flow_method</t>
+        </is>
+      </c>
+      <c r="B67" s="290" t="inlineStr">
+        <is>
+          <t>QUICK</t>
+        </is>
+      </c>
+      <c r="C67" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="116" t="inlineStr">
+        <is>
+          <t>QUICK = debit unitaire L/s/100m (B57). DARCY = calcul k*i*d*L*coef capture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="160" t="inlineStr">
+        <is>
+          <t>Foundation_darcy_scenario</t>
+        </is>
+      </c>
+      <c r="B68" s="290" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="C68" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D68" s="116" t="inlineStr">
+        <is>
+          <t>LOW / BASE / HIGH pour la methode DARCY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="160" t="inlineStr">
+        <is>
+          <t>k_low_m_per_s</t>
+        </is>
+      </c>
+      <c r="B69" s="291" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="C69" s="116" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="D69" s="116" t="inlineStr">
+        <is>
+          <t>Conductivite hydraulique faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="160" t="inlineStr">
+        <is>
+          <t>k_base_m_per_s</t>
+        </is>
+      </c>
+      <c r="B70" s="291" t="n">
+        <v>5e-06</v>
+      </c>
+      <c r="C70" s="116" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="D70" s="116" t="inlineStr">
+        <is>
+          <t>Conductivite hydraulique de base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="160" t="inlineStr">
+        <is>
+          <t>k_high_m_per_s</t>
+        </is>
+      </c>
+      <c r="B71" s="291" t="n">
+        <v>2e-05</v>
+      </c>
+      <c r="C71" s="116" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="D71" s="116" t="inlineStr">
+        <is>
+          <t>Conductivite hydraulique elevee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="160" t="inlineStr">
+        <is>
+          <t>i_low</t>
+        </is>
+      </c>
+      <c r="B72" s="249" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C72" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D72" s="116" t="inlineStr">
+        <is>
+          <t>Gradient hydraulique faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="160" t="inlineStr">
+        <is>
+          <t>i_base</t>
+        </is>
+      </c>
+      <c r="B73" s="249" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C73" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D73" s="116" t="inlineStr">
+        <is>
+          <t>Gradient hydraulique de base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="160" t="inlineStr">
+        <is>
+          <t>i_high</t>
+        </is>
+      </c>
+      <c r="B74" s="249" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C74" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D74" s="116" t="inlineStr">
+        <is>
+          <t>Gradient hydraulique eleve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="160" t="inlineStr">
+        <is>
+          <t>d_eff_low_m</t>
+        </is>
+      </c>
+      <c r="B75" s="249" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C75" s="116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D75" s="116" t="inlineStr">
+        <is>
+          <t>Epaisseur captee faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="160" t="inlineStr">
+        <is>
+          <t>d_eff_base_m</t>
+        </is>
+      </c>
+      <c r="B76" s="249" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D76" s="116" t="inlineStr">
+        <is>
+          <t>Epaisseur captee de base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="160" t="inlineStr">
+        <is>
+          <t>d_eff_high_m</t>
+        </is>
+      </c>
+      <c r="B77" s="249" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C77" s="116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D77" s="116" t="inlineStr">
+        <is>
+          <t>Epaisseur captee elevee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="160" t="inlineStr">
+        <is>
+          <t>capture_factor_low</t>
+        </is>
+      </c>
+      <c r="B78" s="249" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C78" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D78" s="116" t="inlineStr">
+        <is>
+          <t>Facteur de captage faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="160" t="inlineStr">
+        <is>
+          <t>capture_factor_base</t>
+        </is>
+      </c>
+      <c r="B79" s="249" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D79" s="116" t="inlineStr">
+        <is>
+          <t>Facteur de captage de base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="160" t="inlineStr">
+        <is>
+          <t>capture_factor_high</t>
+        </is>
+      </c>
+      <c r="B80" s="249" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C80" s="116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D80" s="116" t="inlineStr">
+        <is>
+          <t>Facteur de captage eleve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_darcy_low_m3s</t>
+        </is>
+      </c>
+      <c r="B81" s="249">
+        <f>B55*B69*B72*B75*B78</f>
+        <v/>
+      </c>
+      <c r="C81" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D81" s="116" t="inlineStr">
+        <is>
+          <t>Q = L * k * i * d_eff * coef_capture (scenario LOW).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_darcy_base_m3s</t>
+        </is>
+      </c>
+      <c r="B82" s="249">
+        <f>B55*B70*B73*B76*B79</f>
+        <v/>
+      </c>
+      <c r="C82" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D82" s="116" t="inlineStr">
+        <is>
+          <t>Q = L * k * i * d_eff * coef_capture (scenario BASE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_darcy_high_m3s</t>
+        </is>
+      </c>
+      <c r="B83" s="249">
+        <f>B55*B71*B74*B77*B80</f>
+        <v/>
+      </c>
+      <c r="C83" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D83" s="116" t="inlineStr">
+        <is>
+          <t>Q = L * k * i * d_eff * coef_capture (scenario HIGH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_darcy_selected_m3s</t>
+        </is>
+      </c>
+      <c r="B84" s="249">
+        <f>IF(OR(UPPER(TRIM(B68))="LOW",UPPER(TRIM(B68))="BAS"),B81,IF(UPPER(TRIM(B68))="HIGH",B83,B82))</f>
+        <v/>
+      </c>
+      <c r="C84" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D84" s="116" t="inlineStr">
+        <is>
+          <t>Selection scenario LOW/BASE/HIGH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="160" t="inlineStr">
+        <is>
+          <t>Q_foundation_selected_method_m3s</t>
+        </is>
+      </c>
+      <c r="B85" s="249">
+        <f>IF(OR(UPPER(TRIM(B67))="DARCY",UPPER(TRIM(B67))="D"),B84,B57)</f>
+        <v/>
+      </c>
+      <c r="C85" s="116" t="inlineStr">
+        <is>
+          <t>m3/s</t>
+        </is>
+      </c>
+      <c r="D85" s="116" t="inlineStr">
+        <is>
+          <t>Debit retenu par methode (QUICK ou DARCY).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="160" t="inlineStr">
+        <is>
+          <t>V_foundation_selected_event_m3</t>
+        </is>
+      </c>
+      <c r="B86" s="249">
+        <f>B85*B52*60</f>
+        <v/>
+      </c>
+      <c r="C86" s="116" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D86" s="116" t="inlineStr">
+        <is>
+          <t>Volume evenement associe au debit retenu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add non-intrusive level mapping and aval-routing explanation tab
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Pertes_singulieres_detail" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Analyse_duree" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Aval_manhole_sync" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Liaison_niveaux" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="A_wetwell" hidden="0" function="0" vbProcedure="0">Pump_Sizing!$E$39</definedName>
@@ -517,7 +518,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="292">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1346,6 +1347,11 @@
     <xf numFmtId="11" fontId="8" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="17" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -31060,4 +31066,376 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="117" min="1" max="1"/>
+    <col width="24" customWidth="1" style="117" min="2" max="2"/>
+    <col width="22" customWidth="1" style="117" min="3" max="3"/>
+    <col width="56" customWidth="1" style="117" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="270" t="inlineStr">
+        <is>
+          <t>Liaison des niveaux (sans modifier les valeurs existantes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="231" t="inlineStr">
+        <is>
+          <t>Cet onglet est en lecture/formules uniquement. Il ne change aucun parametre des onglets Inputs, Pump_Sizing, Routing ou Aval_manhole_sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="292" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="B4" s="292" t="inlineStr">
+        <is>
+          <t>Cellule source</t>
+        </is>
+      </c>
+      <c r="C4" s="292" t="inlineStr">
+        <is>
+          <t>Valeur liee</t>
+        </is>
+      </c>
+      <c r="D4" s="292" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="293" t="inlineStr">
+        <is>
+          <t>Wetwell_invert_m (fond du puisard)</t>
+        </is>
+      </c>
+      <c r="B5" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B40</t>
+        </is>
+      </c>
+      <c r="C5" s="294">
+        <f>Inputs!$B$40</f>
+        <v/>
+      </c>
+      <c r="D5" s="293" t="inlineStr">
+        <is>
+          <t>Cote geometrique du fond (structure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="293" t="inlineStr">
+        <is>
+          <t>Pump_ON_1_m (marche pompe 1)</t>
+        </is>
+      </c>
+      <c r="B6" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B19</t>
+        </is>
+      </c>
+      <c r="C6" s="294">
+        <f>Inputs!$B$19</f>
+        <v/>
+      </c>
+      <c r="D6" s="293" t="inlineStr">
+        <is>
+          <t>Niveau de demarrage de la pompe 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="293" t="inlineStr">
+        <is>
+          <t>Pump_OFF_1_m (arret pompe 1)</t>
+        </is>
+      </c>
+      <c r="B7" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B20</t>
+        </is>
+      </c>
+      <c r="C7" s="294">
+        <f>Inputs!$B$20</f>
+        <v/>
+      </c>
+      <c r="D7" s="293" t="inlineStr">
+        <is>
+          <t>Niveau d arret de la pompe 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="293" t="inlineStr">
+        <is>
+          <t>Niveau d exploitation du puisard</t>
+        </is>
+      </c>
+      <c r="B8" s="286" t="inlineStr">
+        <is>
+          <t>Pump_Sizing!B6</t>
+        </is>
+      </c>
+      <c r="C8" s="294">
+        <f>Pump_Sizing!$B$6</f>
+        <v/>
+      </c>
+      <c r="D8" s="293" t="inlineStr">
+        <is>
+          <t>Dans votre fichier: moyenne entre Inputs!B19 et Inputs!B20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="293" t="inlineStr">
+        <is>
+          <t>Niveau eau ruisseau (reference aval)</t>
+        </is>
+      </c>
+      <c r="B9" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B12</t>
+        </is>
+      </c>
+      <c r="C9" s="294">
+        <f>Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="D9" s="293" t="inlineStr">
+        <is>
+          <t>Utilise pour la charge statique dans Pump_Sizing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="293" t="inlineStr">
+        <is>
+          <t>Charge statique calculee</t>
+        </is>
+      </c>
+      <c r="B10" s="286" t="inlineStr">
+        <is>
+          <t>Pump_Sizing!B19</t>
+        </is>
+      </c>
+      <c r="C10" s="294">
+        <f>Pump_Sizing!$B$19</f>
+        <v/>
+      </c>
+      <c r="D10" s="293">
+        <f>MAX(0, Niveau ruisseau - Niveau exploitation).</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="278" t="inlineStr">
+        <is>
+          <t>Diagnostics derives (controle de coherence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="287" t="inlineStr">
+        <is>
+          <t>Indicateur</t>
+        </is>
+      </c>
+      <c r="B13" s="287" t="inlineStr">
+        <is>
+          <t>Formule</t>
+        </is>
+      </c>
+      <c r="C13" s="287" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="D13" s="287" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="293" t="inlineStr">
+        <is>
+          <t>ON &gt; OFF ?</t>
+        </is>
+      </c>
+      <c r="B14" s="286">
+        <f>C6&gt;C7</f>
+        <v/>
+      </c>
+      <c r="C14" s="285">
+        <f>IF(C6&gt;C7,"OK","A REVOIR")</f>
+        <v/>
+      </c>
+      <c r="D14" s="293" t="inlineStr">
+        <is>
+          <t>Pour un controle standard, ON devrait etre &gt; OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="293" t="inlineStr">
+        <is>
+          <t>Submergence a OFF (m)</t>
+        </is>
+      </c>
+      <c r="B15" s="286">
+        <f>C7-C5</f>
+        <v/>
+      </c>
+      <c r="C15" s="294">
+        <f>C7-C5</f>
+        <v/>
+      </c>
+      <c r="D15" s="293" t="inlineStr">
+        <is>
+          <t>Profondeur d eau au niveau OFF au-dessus du fond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="293" t="inlineStr">
+        <is>
+          <t>Submergence a ON (m)</t>
+        </is>
+      </c>
+      <c r="B16" s="286">
+        <f>C6-C5</f>
+        <v/>
+      </c>
+      <c r="C16" s="294">
+        <f>C6-C5</f>
+        <v/>
+      </c>
+      <c r="D16" s="293" t="inlineStr">
+        <is>
+          <t>Profondeur d eau au niveau ON au-dessus du fond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="293" t="inlineStr">
+        <is>
+          <t>Bande ON-OFF (m)</t>
+        </is>
+      </c>
+      <c r="B17" s="286">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="C17" s="294">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="D17" s="293" t="inlineStr">
+        <is>
+          <t>Hysteresis de commande (plus grand = moins de cycles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="293" t="inlineStr">
+        <is>
+          <t>Niveau exploitation - OFF (m)</t>
+        </is>
+      </c>
+      <c r="B18" s="286">
+        <f>C8-C7</f>
+        <v/>
+      </c>
+      <c r="C18" s="294">
+        <f>C8-C7</f>
+        <v/>
+      </c>
+      <c r="D18" s="293" t="inlineStr">
+        <is>
+          <t>Ecart entre niveau exploitation et niveau OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="293" t="inlineStr">
+        <is>
+          <t>Niveau exploitation - ON (m)</t>
+        </is>
+      </c>
+      <c r="B19" s="286">
+        <f>C8-C6</f>
+        <v/>
+      </c>
+      <c r="C19" s="294">
+        <f>C8-C6</f>
+        <v/>
+      </c>
+      <c r="D19" s="293" t="inlineStr">
+        <is>
+          <t>Ecart entre niveau exploitation et niveau ON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="278" t="inlineStr">
+        <is>
+          <t>A quoi sert Aval_manhole_sync ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="293" t="inlineStr">
+        <is>
+          <t>1) Ce bloc route le volume/niveau dans le regard aval APRES le poste de pompage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="293" t="inlineStr">
+        <is>
+          <t>2) A chaque pas: V_fin = MAX(0, V_debut + (Q_in - Q_out)*dt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="293" t="inlineStr">
+        <is>
+          <t>3) Q_in provient de Routing!M (debit pompe effectif) et Q_out provient de la courbe niveau-debit (colonnes J:K du meme onglet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="293" t="inlineStr">
+        <is>
+          <t>4) Le tableau calcule ensuite Vmax, V requis avec facteur de securite, hauteur requise et verification du niveau max admissible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="293" t="inlineStr">
+        <is>
+          <t>5) Si "Verification_niv" = FAIL, le regard aval depasse le niveau admissible choisi (B12).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sync workbook from commit 8aa4e7e
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
+++ b/engineering/stormwater-pumping/PostPompagePluvial_Meta_TRAVAIL_maison_FR.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Pertes_singulieres_detail" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Analyse_duree" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Aval_manhole_sync" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Liaison_niveaux" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="A_wetwell" hidden="0" function="0" vbProcedure="0">Pump_Sizing!$E$39</definedName>
@@ -517,7 +518,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="292">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1346,6 +1347,11 @@
     <xf numFmtId="11" fontId="8" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="17" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -31060,4 +31066,376 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="117" min="1" max="1"/>
+    <col width="24" customWidth="1" style="117" min="2" max="2"/>
+    <col width="22" customWidth="1" style="117" min="3" max="3"/>
+    <col width="56" customWidth="1" style="117" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="270" t="inlineStr">
+        <is>
+          <t>Liaison des niveaux (sans modifier les valeurs existantes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="231" t="inlineStr">
+        <is>
+          <t>Cet onglet est en lecture/formules uniquement. Il ne change aucun parametre des onglets Inputs, Pump_Sizing, Routing ou Aval_manhole_sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="292" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+      <c r="B4" s="292" t="inlineStr">
+        <is>
+          <t>Cellule source</t>
+        </is>
+      </c>
+      <c r="C4" s="292" t="inlineStr">
+        <is>
+          <t>Valeur liee</t>
+        </is>
+      </c>
+      <c r="D4" s="292" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="293" t="inlineStr">
+        <is>
+          <t>Wetwell_invert_m (fond du puisard)</t>
+        </is>
+      </c>
+      <c r="B5" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B40</t>
+        </is>
+      </c>
+      <c r="C5" s="294">
+        <f>Inputs!$B$40</f>
+        <v/>
+      </c>
+      <c r="D5" s="293" t="inlineStr">
+        <is>
+          <t>Cote geometrique du fond (structure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="293" t="inlineStr">
+        <is>
+          <t>Pump_ON_1_m (marche pompe 1)</t>
+        </is>
+      </c>
+      <c r="B6" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B19</t>
+        </is>
+      </c>
+      <c r="C6" s="294">
+        <f>Inputs!$B$19</f>
+        <v/>
+      </c>
+      <c r="D6" s="293" t="inlineStr">
+        <is>
+          <t>Niveau de demarrage de la pompe 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="293" t="inlineStr">
+        <is>
+          <t>Pump_OFF_1_m (arret pompe 1)</t>
+        </is>
+      </c>
+      <c r="B7" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B20</t>
+        </is>
+      </c>
+      <c r="C7" s="294">
+        <f>Inputs!$B$20</f>
+        <v/>
+      </c>
+      <c r="D7" s="293" t="inlineStr">
+        <is>
+          <t>Niveau d arret de la pompe 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="293" t="inlineStr">
+        <is>
+          <t>Niveau d exploitation du puisard</t>
+        </is>
+      </c>
+      <c r="B8" s="286" t="inlineStr">
+        <is>
+          <t>Pump_Sizing!B6</t>
+        </is>
+      </c>
+      <c r="C8" s="294">
+        <f>Pump_Sizing!$B$6</f>
+        <v/>
+      </c>
+      <c r="D8" s="293" t="inlineStr">
+        <is>
+          <t>Dans votre fichier: moyenne entre Inputs!B19 et Inputs!B20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="293" t="inlineStr">
+        <is>
+          <t>Niveau eau ruisseau (reference aval)</t>
+        </is>
+      </c>
+      <c r="B9" s="286" t="inlineStr">
+        <is>
+          <t>Inputs!B12</t>
+        </is>
+      </c>
+      <c r="C9" s="294">
+        <f>Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="D9" s="293" t="inlineStr">
+        <is>
+          <t>Utilise pour la charge statique dans Pump_Sizing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="293" t="inlineStr">
+        <is>
+          <t>Charge statique calculee</t>
+        </is>
+      </c>
+      <c r="B10" s="286" t="inlineStr">
+        <is>
+          <t>Pump_Sizing!B19</t>
+        </is>
+      </c>
+      <c r="C10" s="294">
+        <f>Pump_Sizing!$B$19</f>
+        <v/>
+      </c>
+      <c r="D10" s="293">
+        <f>MAX(0, Niveau ruisseau - Niveau exploitation).</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="278" t="inlineStr">
+        <is>
+          <t>Diagnostics derives (controle de coherence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="287" t="inlineStr">
+        <is>
+          <t>Indicateur</t>
+        </is>
+      </c>
+      <c r="B13" s="287" t="inlineStr">
+        <is>
+          <t>Formule</t>
+        </is>
+      </c>
+      <c r="C13" s="287" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="D13" s="287" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="293" t="inlineStr">
+        <is>
+          <t>ON &gt; OFF ?</t>
+        </is>
+      </c>
+      <c r="B14" s="286">
+        <f>C6&gt;C7</f>
+        <v/>
+      </c>
+      <c r="C14" s="285">
+        <f>IF(C6&gt;C7,"OK","A REVOIR")</f>
+        <v/>
+      </c>
+      <c r="D14" s="293" t="inlineStr">
+        <is>
+          <t>Pour un controle standard, ON devrait etre &gt; OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="293" t="inlineStr">
+        <is>
+          <t>Submergence a OFF (m)</t>
+        </is>
+      </c>
+      <c r="B15" s="286">
+        <f>C7-C5</f>
+        <v/>
+      </c>
+      <c r="C15" s="294">
+        <f>C7-C5</f>
+        <v/>
+      </c>
+      <c r="D15" s="293" t="inlineStr">
+        <is>
+          <t>Profondeur d eau au niveau OFF au-dessus du fond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="293" t="inlineStr">
+        <is>
+          <t>Submergence a ON (m)</t>
+        </is>
+      </c>
+      <c r="B16" s="286">
+        <f>C6-C5</f>
+        <v/>
+      </c>
+      <c r="C16" s="294">
+        <f>C6-C5</f>
+        <v/>
+      </c>
+      <c r="D16" s="293" t="inlineStr">
+        <is>
+          <t>Profondeur d eau au niveau ON au-dessus du fond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="293" t="inlineStr">
+        <is>
+          <t>Bande ON-OFF (m)</t>
+        </is>
+      </c>
+      <c r="B17" s="286">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="C17" s="294">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="D17" s="293" t="inlineStr">
+        <is>
+          <t>Hysteresis de commande (plus grand = moins de cycles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="293" t="inlineStr">
+        <is>
+          <t>Niveau exploitation - OFF (m)</t>
+        </is>
+      </c>
+      <c r="B18" s="286">
+        <f>C8-C7</f>
+        <v/>
+      </c>
+      <c r="C18" s="294">
+        <f>C8-C7</f>
+        <v/>
+      </c>
+      <c r="D18" s="293" t="inlineStr">
+        <is>
+          <t>Ecart entre niveau exploitation et niveau OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="293" t="inlineStr">
+        <is>
+          <t>Niveau exploitation - ON (m)</t>
+        </is>
+      </c>
+      <c r="B19" s="286">
+        <f>C8-C6</f>
+        <v/>
+      </c>
+      <c r="C19" s="294">
+        <f>C8-C6</f>
+        <v/>
+      </c>
+      <c r="D19" s="293" t="inlineStr">
+        <is>
+          <t>Ecart entre niveau exploitation et niveau ON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="278" t="inlineStr">
+        <is>
+          <t>A quoi sert Aval_manhole_sync ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="293" t="inlineStr">
+        <is>
+          <t>1) Ce bloc route le volume/niveau dans le regard aval APRES le poste de pompage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="293" t="inlineStr">
+        <is>
+          <t>2) A chaque pas: V_fin = MAX(0, V_debut + (Q_in - Q_out)*dt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="293" t="inlineStr">
+        <is>
+          <t>3) Q_in provient de Routing!M (debit pompe effectif) et Q_out provient de la courbe niveau-debit (colonnes J:K du meme onglet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="293" t="inlineStr">
+        <is>
+          <t>4) Le tableau calcule ensuite Vmax, V requis avec facteur de securite, hauteur requise et verification du niveau max admissible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="293" t="inlineStr">
+        <is>
+          <t>5) Si "Verification_niv" = FAIL, le regard aval depasse le niveau admissible choisi (B12).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>